<commit_message>
Update topic news feed (daily)
</commit_message>
<xml_diff>
--- a/data/daily/topic_feeds_daily.xlsx
+++ b/data/daily/topic_feeds_daily.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,354 +470,354 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ETS Nigeria Conflict Situation Report #109: January 2026 - ReliefWeb</t>
+          <t>Enhanced Free Trade Agreement with Switzerland round update - GOV.UK</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:33:09 GMT</t>
+          <t>Mon, 02 Feb 2026 18:05:45 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOY2RLR1BHd1ZqN1d2c05HS0luYXYyUTB2ZGVhaFp6WFhmVW1yekJtY29oakx1OXc4VjA4bjVNUVdMX09YSldURkVOTjdPaWlmZE02S0xpWVVQVlRHUDZXd0VoYXZtZTFoU0V0VHV1SXBIRnM4aV94UUd2VkdOMGJfTGFBTV9pdDRWMldEcW5HNDl6UXV3b0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPNm9tY21mV1p0R0tWX29YZXpfaU1tOGdWWnd3Q2IxMDJKdFdCNklhOEZnVnlydVZEWHNVNTJWN3c0Y2Y1WVVzd1VCaXdPZkh1N2UxNkloTVduV0U0aThIOUlYQ2V1S3kyc3ZwYXhDMzcxQW5YbkljVkw4RGEyOEZvMFFGR09KNFhCRTQtcjhPQUt4cVVCYzlPdF9R?oc=5</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46055.39802083333</v>
+        <v>46055.75399305556</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Logistics Manager Magazine February 2026 - Logistics Manager</t>
+          <t>Fox Williams cited in Treasury Select Committee report on AI regulation - Fox Williams</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:00:25 GMT</t>
+          <t>Mon, 02 Feb 2026 15:59:28 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE5WM3c1Um9FY0RtamoxcENreVJvWUpQbWl0ODFqb0VUX0tqTk8xTVM4SmRkc21FLWJJV3pnNVhUcDlUbU5CRHpNWGhNcjRidTVHZ0Qxd09zaWFZV3NIc01mWlpYQ1ZVZ2dYTUtiMEt5ZGRCWVc3dTl2c1pNZ3ozVEE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxONUticHMyRF85OV9QcFRDQm5LV0YwTDc2c2RjZjRFcnpmUXJIcXRVWlIwSWpEdXNpbkp5eUMyZWh2UHNXbHFZcHlIZDJBWkJoQl96ZDAtdUtSc0xodUVGSzh6Q1pDTFdlal9RTmlEUVRZcjRMWXo4TE1feVlCaFJ6RExTR1ZYWHJZRllZMzZJaFhKTy0ydmVIX201Y2pPcHdIZUtVV3BzYm03YzIwbUQzYg?oc=5</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>46055.50028935185</v>
+        <v>46055.66629629629</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UK manufacturers recalibrate trade strategies as tariffs bite - Relocate magazine</t>
+          <t>US jobs report delayed again amid government shutdown - The Guardian</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:43:42 GMT</t>
+          <t>Mon, 02 Feb 2026 19:46:00 GMT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPNVhoOENKNGhOeVEtZTU1RlB5ZVZ3Zm1Obkw3Xzg3MVFXUnFkZ1ozZmJKZUZKSGhyNmNtMGZfTjRsOHFkLUxUTWMyUzRBbGx3RTRFZU5DQ1ZCODdZSXRTa0V6WmdyeUVqSHA4amw2NEtHNXNmVG1wdEFqOWRPSWlDei1Zcm10a1BvbzQwUi1kb3F6ZWdZeFNXbmV4RS1Gcm9YSkpmUmZBcUw4QnM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxQX1ZZelJzVEM5Q2gyb1dsa1dfSjdScEdlRTA0azlsdVU1N3FXNDdmWVd5b3E2eDFYMFpISXYtVEV6azA4b1JBTjJacFViai1SYWlCcWxLZ3hYQmNhMEU4MnpwQXRscWlacVRaWXJnbGNua0RFc2ZBWDFqbVk5cmUzWGwwQUUtbnY5bUp6TDB0WFV0dXkxYUE?oc=5</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>46055.44701388889</v>
+        <v>46055.82361111111</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Services - GIMA Day Conference 2026: the future of the supply chain for garden products - gardenforum.co.uk</t>
+          <t>Briefing: asylum seeker social care costs in local authorities - The TaxPayers' Alliance</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:04:40 GMT</t>
+          <t>Mon, 02 Feb 2026 07:52:30 GMT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPU3VFMUNRR1duajV0UmZPN3VTeklQYUF6VXlmbmc0RmdXOXpseW5Cd1FTdnBLNS1nQmoxbGNOQjEwWkp2RThUQUZLUlUyYVJwVnhKUFpzV1RPUkZwUDJHYTlpSnltdFNUaXlwT1cwMUpRVnFiVVhLcHFmczVMRUNmV19vbUZPWlg1SllsSTAzQm5HeG05X0NXWk1UVjlDQTd2NUlzaExVU2tLTlpYaHIzM2ZLLXpEQndfQmM4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPWGdja0oxNFNLVHVRc09JckljX182MU42Y0d3eGczU0xnM2hsNUUzd1c4Ykd2SkNzQmVzY1VQcmtEVHIxUWljelRpMXlzbUVLbFVQdkcxZHFjWnZlcnZaNkh2X0MxS3JtX2k2UGV3aXU5MWZpUzNnZElPdFEwQVU3czhwRmNnamJYRXRjNW9fN013b3Z6N0tF?oc=5</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>46055.50324074074</v>
+        <v>46055.328125</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Price of consumer goods could surge as shipping costs soar, industry body says - The Guardian</t>
+          <t>New report finds quarter of young Scots fear they will fail in life - Daily Record</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 13:00:00 GMT</t>
+          <t>Tue, 03 Feb 2026 04:30:00 GMT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNM2ZMdGRNWlRFaVVqVHg2Q0Q3X0c1Um5uRFEzRnJselR5czM5OXJZdHdCOVpnUGxtbXo3VUlTekowNkZMaEgyeEtBeDVDUEZfSXhyZG80NlQ4bFp1cnFwTVdCdURyRnk5Zzc0N2doM1BqSFBIY25Jb2dMdUhCclVTZV93XzNsQm9VN1R3VFY3ejB6eVQ4M1ZGRmI4SV9FdEhCcXI0VEdIQVAzVjV6bHBDdmNwZzlzd2c5OVpuNmVaa09vWmdFcjBKQkJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxNd0pXZ1JVcVQwQVpsUGIyYWgwbXJXRTVVVF9IYTlrenMtRzJkci0wczJURllGeFdJc2Q5NUpYVUFpUG5UYWNwZEhmNVZCLWh5TEp2Y1lwTV9sZHZIbkxoMmJPY1hMTDRNOUotSVdMOUFKZk1xX3BVQ3JNcDhWQ3psTjNJTno2bjA4VjFnVnhBMG5jUdIBlwFBVV95cUxNN3FBR1hkWWhVZk01aWlsTGIxd3V5V2FkTTRlMGlULTNMOHlzMlFWZjJWbG5DU0tUbl9LVVBHMFhDX0NwUkl3cng1YWNWMG5XZGZCWm1fU0xIeG1PZWFwY01ENEJKLWY0X2poOUtpU0lqM2lqMVhKMndXVjUyNGZmak51ZEExeDNCUmNGWFpFN2xudkxGTi0w?oc=5</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>46054.54166666666</v>
+        <v>46056.1875</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>China cuts tariffs on Scotch whisky - The Drinks Business</t>
+          <t>Opinion: The report the government didn't want you to read about climate decline - Eastern Daily Press</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:56:37 GMT</t>
+          <t>Tue, 03 Feb 2026 06:00:00 GMT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxPblMwMm5fMVJQejYzOWRYQ1BWWDhud0tfeTlIdnEzUEZYanRMbWdhQlhVNnprRGs0SVdjNjJtb2p4SUN1emU2ZnZBdl9HTVV6aFFvSUV4bWtsYTVnWjMyNzM3N0xQcVRWelpObUVQb0tUaE0tdkR5SGduMGhXWnpZWWF6SXU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNUGZ6R240am5jMWlPN2t6N0k0cVVZQU1rVmVMUDJaWEJuSDdXV2c1UWU1UUoxNTVwc0RtLWE3eVJTdDNzSW5WQmVxVUsxcjdaQ1JNcFIyQ2Z5UlRsZ0VZb2hxY1RPOFJHNzhxSV9yNFluRlRvenptbU9NWEVOUWtlRFdHTnBxUzFKa0pWcDFR?oc=5</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>46055.4559837963</v>
+        <v>46056.25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>NPA host Agricultural Supply Chain Adjudicator in Lincolnshire - National Pig Association</t>
+          <t>Thriving Kids Advisory Group Final Report - MBS Online</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:49:27 GMT</t>
+          <t>Mon, 02 Feb 2026 22:47:12 GMT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQOFBxVjc5ZFRKY2h4WHFMcmhnbWVBckZHNlpfVk9PVUhhREtMUldwMzd6c1hJUnZPZVRRRklRa1hHek14SHVvWGo0YmdVM1hxQ2g4cWFoNVo0Q2tRc0FUeUNsSnFFc3hXcnRqU2oxMTB4RmU4QkVWSFIxN2kyWjFhLVhPQk4xS3Q2Qk0wd1hXeVFxN1ZLVkxBbmhvVHZFTzJxV2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxQSU55MTVrdlV5c3kyTDhpTlBoM1J4UVlXSzZ1ajFiV2FFRmdtZEV1TGV3eUZvSWxNTFdRMjRiY1Jreko5WWZDVmQ1X09ndjEyUmZxQ19EWU1zXzlxdkZ5T0VjMnd2YnNLbEFMWWtjNC13MlN4ajVTM09KY0pjdHJVdlBkMXlhN2xMY0VHTnZ6cDlzYjJ5R2VCbEhmREk3UnZ2SkpEYw?oc=5</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>46055.45100694444</v>
+        <v>46055.94944444444</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Columbia Group appoints Prevention at Sea as compliance partner and rolls out MORSE platform across the fleet - shipmanagementinternational.com</t>
+          <t>Migrant encounters at the U.S.-Mexico border are at their lowest level in more than 50 years - Pew Research Center</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:34:37 GMT</t>
+          <t>Mon, 02 Feb 2026 18:55:15 GMT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxObWwwd0JPOVh6Rkp0cmFwckNxZ25TSThzZWtyS0N1dkRGOUV2ODBpUl82djNtZDROVVlmYUNibnpRUW5Cb2pvYnBWRGlLZk1xb2p6YVVqNXdsSWRRRTBFdDdPMWNpZ3JERDlvQzBkQy1qYU0tb2Q0MjQxcm9XZUlpdTc5aWR0OUxnbWV5QS13VDNxdkRMZ00wWm8wVlJENTBRdmZBR0k2dlVnSmNiRnVmZHFzRVktaTNXaU9FZWZ5YkthVHFkUndmWERXdFFYWjk3WU8zUXVFM2NPSlU2OWdDU2FLYXk3Y3NaekE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2gFBVV95cUxQcXUzZzRjaHZIb2g5VVJLZ1RvYktBWm1rdXBWTm45ZlBkbWNOdTRWOFlvWVlBQ1JYV1dXVkVIRWVwY0tmZ29LN0tWdUxEQktDZUlLRHcyaXN2QUFxZ3RRejUtR1NWMHJuX1dBalM2Q1VXMmFfMlUwYUwzTWItYTdRbkxyY2tiVVB4T2c2blR5X1hGWXBKbUttNjhYQUhnOGVhLWlEb091ZDBjcVZMVTg3a3IxSjBwVndTX1E2U0hrcFFFT2laWGdfNE9WeFpfR3ZjeWdKZjhhdktiQQ?oc=5</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>46055.44070601852</v>
+        <v>46055.78836805555</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>The North East’s Green Super Port: 18 months on, the opportunity remains vast - North East Bylines</t>
+          <t>Government report highlights artificial intelligence gains in Kazakhstan - IntelliNews</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:12:00 GMT</t>
+          <t>Mon, 02 Feb 2026 15:37:20 GMT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOamgxNERESWJlUy11VUpyMHBVazQzM0tMUXpNRzY3UTk5bXBoV0x2bVZUMkxaUFl1YUFrS3NldGFfY2xuNy1jcjB0amc2UFR0cGlqWWlyQTFpVEVadkY4akJuU2FTeEF1M0FfMXgxejlrbVJvZDhpVFZEcVlVY1N4MFpBaGZnMm5ObmtxemxDWk41V0h4STExZ00wbEhuVWtJQkpha0pHLTI1VG9EdG5wXzBqbm5zY3E4dmpzbUlRekY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxORGNzMl93aTlJdnFiczhjYnJNOXZMd3pNQlotRFRmS2RBd3hibUhieGlQTHR1MHY1eVpPQUtlVGEzM01KclZERFBPTkl5YU45X1JGTkNOaUZCTlhYdEVwT09OZFB5RURoUjN0TWxnbXk5V2J0dHJaQkc4VGVaZmttcGFwUWN2M3dUT2xYUGQyaFVYX0piM3J1NVFxWTZsWmtickt5dWJwMUpNWEZl?oc=5</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>46055.34166666667</v>
+        <v>46055.65092592593</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mapletree on how European logistics is gaining momentum - Private Equity Real Estate | PERE</t>
+          <t>Economy update: Seven Labubu stores to open in Britain after Keir Starmer's China visit - GB News</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 02:02:52 GMT</t>
+          <t>Mon, 02 Feb 2026 14:01:53 GMT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQbF9UQXJKSXljNU5GeW9JZmpVZ0ZobUNnTFF5bVFxanRIam4xX2lNMENFeTVJT1Z2WHF1bXI3WHphYXhfd0VQNWx1Z25UVy1WNkFKY0ZmY3hfYTAyYVhJanRnSW44M09CZ2lOcmRIc2czTnY2OVc3UlhFWjc5VGtSYng4QzNxbExj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE1kbUtPWWFJNVlGT2YyTU9OWEl0Y3F0SDQwWE9ELS1EXy1fd2xTQ3JNZEhiN0RENWg2RGxDZ2J6bGxBRGZ2NldxUkFUMFdRRlctMXZoY2R0UnB2RjhGSlM3cEJtOHB5TVBLRUhpbTlNdkhWNzA4SEtB?oc=5</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>46055.08532407408</v>
+        <v>46055.58464120371</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Current_Affairs</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(geopolitics OR migration OR economy OR conflict OR legislation OR terrorism OR disinformation OR misinformation OR government OR policy OR regulation) AND (briefing OR analysis OR update OR report)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Geopolitics is rewriting freight rules - Air Cargo Week</t>
+          <t>UK’s former US ambassador faces scrutiny over Epstein ties, leaked briefing - South China Morning Post</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:50:44 GMT</t>
+          <t>Mon, 02 Feb 2026 15:59:12 GMT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBCSGVRWDFSV3p6eDNUb05PME9ieHF4TkJ2azVoNFUxcDU5WDhFemd3S0xEWmVadXY4R3M1OXdVR0RyQUo1cGhmTlRyN19idnlCbHNUY194My11ZUNKcHhoWnBfRkRNTVprbGZLc1pqLUpsdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxPUkp2RzlBQ1hqN3RUY1RpS21EZlRoakx3ZXlaZWlxS2ZUMTdfZ0RDQnZkNm9oT3lwYzBYMUJLNl95Q3JWOVFxa080eEVpcUFheV9SSlVGWFUwbFhnTVczSWFKMUt0bk9mc21rbDZfVF9jWVcxU2hxRnU2dEVyN1hUc1J3NkJwbDd1OTExa0c4NkJjZ2VpbWlKZWYtM3BIYmczVnZuNXVrb0N1QVVkNlJkS0xlZGZFZHVVUGx3TE5zLUFHOV9pampaTFVn0gHKAUFVX3lxTFBVSElBNWxvdHZQSVZvNGt6eWJ4TnRRMW5OcEpITlVRZEJQZjE1eWJDVEppTW9pdHlZY1VpWkxjQlMtemJVWTN3SzZielBrcE5LU3JDVkt4NVA0aVdBLUl3d0c0SzRJUkt4ODJkRHBWMFRTaWY2TUV6ZF9BOXh4b2d5cDJxWUlBei1jeXBIYXBnUEF3YXlhUlRlaU44YXFIZXB2VkJkLUJsMmw2LWhveUp0WURTVGU0cGZJNHlIWklYc0tEOEJMeDVBRnc?oc=5</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>46055.53523148148</v>
+        <v>46055.66611111111</v>
       </c>
     </row>
     <row r="13">
@@ -833,24 +833,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Apollo appoints Valor as asset manager for logistics portfolio - Logistics Manager</t>
+          <t>Hope and uncertainty as India and US strike long-delayed trade deal - BBC</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:21:00 GMT</t>
+          <t>Tue, 03 Feb 2026 06:29:43 GMT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxOUUx3a255dUZramdIYndNZmxSMGkwVS1fSy12dW5FWUY5d1ltV0RGbF9jRjdBdldRVXA5RW1SVm9sWUF3emNaYW5QLU1hOWpfZlluX2dPZkxGQTZGdHMwVEJ1LW9WeWk1dHlZOHhsWkk3bTI1alhXRjkzUmlZdDJlaE56R1hrX2FHQ2VXTll2N3BzOElsSTk4alhrZng?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBoRHZ3eDU2UERBbkZfcHFSSFdicTdPTFdCM2pMQjJORmV6TGFhT3poR2hzamVwN1V1QlF4UDIwMTFDT0gwZUJwb2EyX05Kd1VINnhEdU9fVDIyZw?oc=5</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>46055.43125</v>
+        <v>46056.27063657407</v>
       </c>
     </row>
     <row r="14">
@@ -866,24 +866,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Clarion acquires Mountpark Chartres 2 - Logistics Manager</t>
+          <t>US agrees to drop tariffs after India stops Russian oil purchases - BBC</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:31:48 GMT</t>
+          <t>Mon, 02 Feb 2026 17:55:54 GMT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE9tY2V5UFFHU0pfb0hCa25JNHk5S0JWbXZadk5kU1ZKSWV3QzQtN05HRk5CeHBVeHpQYTdFSVR3UVVIcGVzczJxR2ZEa1dlWjlXcFNaT1E2enVuM0UyUldUai1iU25xSk1PT2NqLUFNWUpUTzI2a043ZHdSYw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1OYXl3VnhHNkQ4QTZEUmpXS0JobDlJeGQ4MTRxbW9xanZvZ2xnY01veXpXNjhBNDR5bWZUUjVoMmdzTHd4dWxxbk1XclNmek9QUzdFTU9sNDIzLVBz?oc=5</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>46055.43875</v>
+        <v>46055.74715277777</v>
       </c>
     </row>
     <row r="15">
@@ -899,24 +899,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wallenius Wilhelmsen starts operating car terminal at Port of Gothenburg - Logistics Manager</t>
+          <t>Modi liberalises Indian tariffs much to chagrin of the left - thecanary.co</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:24:18 GMT</t>
+          <t>Mon, 02 Feb 2026 21:23:15 GMT</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOMzBjYXdWRGJ3QUN4QlgxWjJUeWUtVUxVSzhFbnRDOThwWFRySkJIZjNqUzNMRENVU0gxMzFlVUZqM1Y1dFFJQW9nbTlBQzdxVFdjazJ3XzdxWmgyZEVnblF5NnpscTZueVpuVnotU0Q0aUZTUW81aUM3dkFBSVNSMlMxQnduRUJZekxISnFmRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxNQ05aX2phLTUtaURXdDB6UlZuZU9EWlJXX0s3MTFacURQZnZIdF9tRTI2T0MyOGhIdXJNVC1TbGJNcFBZZkw1T3FrSWtXaHgzcEtIWGJIVW01VTd3dXd5Z3NSbEJKZjQ0M1BEU3A4VXZDaGxOd2JsYzFrNndlV01oQnlqcWlwRzBkTTBkWHRiekxPTFZK?oc=5</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>46055.391875</v>
+        <v>46055.89114583333</v>
       </c>
     </row>
     <row r="16">
@@ -932,24 +932,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Why AI-native execution is the next step for supply chains - Logistics Manager</t>
+          <t>MP asks government about freight-only line amid 'closure by stealth' concerns - Rail Magazine</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:00:55 GMT</t>
+          <t>Tue, 03 Feb 2026 05:02:02 GMT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxOSVEzSlZlTWE4QV9yZlM4QzVlN2pheHJsSjhVSlowVDJUUk9jaGRGT2psZ29OTUdpSENLNkE0VFQ4NjNvdFU4SjFlbXA2WU01M241WEhpMFBTSkxPSmJxTkxHU1pFN3A5SjJ2OEdvNHZRZV91RkZ3bjdDOUYyX2NyLUVaR3NDY3R0UjdtOWlPTDBROFZFZWVN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPc2NSUVZaTlRTVXJBNDNTUFZsazBhdFcxZlI0dXZkSGwzbVBvQ19ybndNamd1Y1NwSXpXTUhJTUNVYllvTzJtWXpLdjNkRmxWdk9uS2hGMlFWSkloLWszM29tdEp4RW5LbmZoS21hb3ZXN05tQnNJcDJHOEp3OXZ5aGJRWERva19HelJJb0RTUUptUklyS2FDZ0xrUm1Yd09Ra0JWQmVObzRKYVFK?oc=5</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>46055.37563657408</v>
+        <v>46056.20974537037</v>
       </c>
     </row>
     <row r="17">
@@ -965,24 +965,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>General Mills: Future-Proofing Sweet Corn Supply Chains - Supply Chain Digital Magazine</t>
+          <t>Grade II listed bridge could reconnect Port Talbot communities - Wales 247</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:36:53 GMT</t>
+          <t>Tue, 03 Feb 2026 06:27:57 GMT</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxPSDNHaERCRzBmS2xTYWNEMUQ3UVdfejZycGRHcExYWHVOZm5LSllMVUE0ZElpcEhkd2czakpfbU5BbnowTFFKN1gyZzBZbkVxdWpVVVEzSFU3UFVfUUNnbERBTUF3VmM3Y2oxMG9KLUp5OUtHQU50alNTTmFCQ0ExVXBfcTNiSDR2eHM1X0JZbXFpQ3dN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOT1JCUC1SQkRNbkhnY2x3RFRsVFFkekI3N2lqaGVLZHY3b2dfUzY5SlpKWnQ4TUpNWHdxeU5hUUtVV2h3eEFDamZCOHZ4anc3bXZ3TFFxVmNZR2NzVjNTb28xODlkbG1BSmZYenFKcTllanhOSXdmUzc1WE1pcUc1aXNILWFUY3JTbkdMRUFFeHkzQ1E?oc=5</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>46055.44228009259</v>
+        <v>46056.26940972222</v>
       </c>
     </row>
     <row r="18">
@@ -998,24 +998,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cargo outlook cools in 2026 as supply chain pressures persist - Air Cargo Week</t>
+          <t>People 'avoid St Peter Port' because of accessibility issues - BBC</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:42:00 GMT</t>
+          <t>Tue, 03 Feb 2026 06:15:03 GMT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPdEo1Y2NzWUg1YW5pbXZqSUFfSC1WX3NCdTIwOS1HUnBCR01XNGIzVmJoZ1hMMWhydnhTeW1JRC01RFZEY2RoMGFHOGV0SmZDVF9IUW5kSGNYRXJsLUVGc05YSW1BYVY0bHktT0NTRGI4QWpxTFZNbXplaEtvT09veUFMT1phTDBXSmw1TExhMGo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTFA5QlNNU2t0Q1JSdmItVU4wUzhEZ2JldGZWbFZLTEVlTG9vM0s0YmRqVndycGJ6RFg5R1pUbXRwT2dXSkg0NXJGZDI3SlM0SXl6RnNSRnczckVsOVdO0gFiQVVfeXFMTVBBOHRyZC1DajNSMUlkLVpma3haLW9vNkg1dW5scHJ5YXNFQ1F5NzVJaGl1YWg3Y3lEcEZDOHZoRlh4UU4xTWNQQmdOcHBYbjRoN21oRnZJdXNaYndaTmJPV1E?oc=5</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>46055.4875</v>
+        <v>46056.26045138889</v>
       </c>
     </row>
     <row r="19">
@@ -1031,24 +1031,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Gold in the age of sanctions: How the Russia-Ukraine war reshaped the global bullion market - New Eastern Europe</t>
+          <t>How Investors Are Reacting To Realty Income (O) Expanding Into Global Logistics With GIC Partnership - Yahoo Finance UK</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:49:35 GMT</t>
+          <t>Tue, 03 Feb 2026 07:09:00 GMT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNRTNnYlFDLVFLdGtpM3pQR0d6TEtJczFsRlZrVEVZa0pKcnBuZXVuNGU4X2Q3a0hackJvYnExOTFfZzFXVTJRcGdRakVoUEV5RGpCNk5zalpUNjRSSXNhTmd4aWd2RTBiTWk3YUpXbVpMZW5GanZaRlJqYWJmbHpmemItZEdvbWhfaHhISmFxNVZRWkxXeEdYMkU3YWlxUDlZRG9FNGJ5WEhDdTd2U25VY3p1djFkazU4aXFYdmQ0d1BabFRHOUxTZlBR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOYVBjTlNZa2pDYS1iQ1pKXzVZYy10UkFZX2FqbWszNGloMlpRSEdoSDRXMUNaY21BeDRvWTlwNkx3ZXFTWVYtcnR4V05BSl9uY1J2X2YxUndPYktIZFNObGg1ekN5dXAtRUJrNmVrUmFINWZYaVo3bFJxQjZJb3VSMEItRlNURURhZnNz?oc=5</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>46055.53443287037</v>
+        <v>46056.29791666667</v>
       </c>
     </row>
     <row r="20">
@@ -1064,24 +1064,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>How AMP8 digital compliance is shaping the water industry - Water Magazine</t>
+          <t>India’s Rupee, Stocks to Get Tariff-Truce Boost, Investors Say - Bloomberg.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 05:05:04 GMT</t>
+          <t>Tue, 03 Feb 2026 07:06:00 GMT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxNT2RfQVZPS1FHeHRURDhWalhPQU43d0RkOGFTTzRxd19BclVwRGtQMlJfUFB5TW5fY294SG13ajVWand6S2Z6a2FCaHFNcTFrQVNJQ0xIbWFOdkRhN2cxbGJ3aVRmVi1tNWt3WUxqUkxuUS1pYk8tWFh6N2ctbXlEYVRQUWd2SFhVNXZiMFVlclgzdkZUU2ZLSEpjdmpuVXpZV2dV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOemVlVDhuUDN6WHNuSGdnZnVfaTRTdXJUQkN6OE16M1lsa2dwRTlNZjhFMkUwbndRZDhCblpSVEc4ZTZFZEk3cjZrUTNNcGd5Q0pQeFV0Y0Q4U21OOXhVQ2dERWJ4NVZGLWpvd2pVMGhDdTBOOWpjWDZtR1ZrclJ6WTZJMGxQTWVuTVdRYWduRUJ0MjJteTNwdUotazJ2amUzOWExenJCeTRTSUhhaEJBSA?oc=5</t>
         </is>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>46055.21185185185</v>
+        <v>46056.29583333333</v>
       </c>
     </row>
     <row r="21">
@@ -1097,24 +1097,24 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EU ready to impose sanctions on Kyrgyzstan — report - Eurasianet</t>
+          <t>South Africa bemoans slow BRICS progress - Fruitnet</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:56:19 GMT</t>
+          <t>Tue, 03 Feb 2026 07:16:45 GMT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTFBWb0tFRFFEc3BtZVhkUV94MWt2MUVzcGNMYmp3eGZHSmk4QmlyTC01U1VjU1JCQU9aM2dsVmMwYzMza1NfRmdHaEJKaGZiOXozMXM5bXVtRVJwb3JmbVhBaF9rRnQ3eTVLQ2lNUVgzcjB2NEI2U3dDX1VXazI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAFBVV95cUxOZ2NHTzE3Znp2OFVmZmgxOXNJSnFpUS1CLTcwVHlnQW5DY2p1NjkxZFBtUnA3cTNDamttWXBjMkljaFFKVXRMbEozeTJNOWRJOEhFQTJBUGRMU2lfVko3WlZtNTJYSUdpSVc4ZlU1MlcxaDI1SnN0eS1OZmdTYzRlNnFGNF84M1BQSkRLaXYtenU1aFIy?oc=5</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="1" t="n">
-        <v>46055.4141087963</v>
+        <v>46056.30329861111</v>
       </c>
     </row>
     <row r="22">
@@ -1130,24 +1130,24 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Port of Tyne appoints new Direct of Innovation - porttechnology.org</t>
+          <t>Diana Shipping secures higher charter rate in extension with Cobelfret - Tradewinds News</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:45:34 GMT</t>
+          <t>Tue, 03 Feb 2026 07:12:31 GMT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNN05iX2doRUpwajRNSDFMVW1MUnU0d2VsOW1fbTdjR0V5Q1VkRzNHWlZwN1BkbV9SLXlYNF9ZNm1wb09YOUR0MU5jNXRTZHpnbWx0bkpsZWZfdTNiUDBOaW9CbWxxcWotZ3M4b2UtM0lseU1IdUpWaWpDaWpYTFRLeENqNjZhcEp4RzBj?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNRlJqZnpUd01zNE52eDRkcGhIZDJhS0lqVVJGNG1ST2c1WVgyUDVWblM1OS0zNWNBbGwweXYtd05NZHFiZHAzUnlzUWdJUmlaWWlxX3NxRlZXeWxDUl9TQVlYV280WUZLNDBUS1BfaXZfaEJNcWZzajBUNk1lTFJ5T0txRHhfZjVTNE1tbEtKci0yZ19qd1ozVkgwMHljMmI1ZklNY05lNlUybjcxdWw0alRmdjRvSzZFeG41ZXR3?oc=5</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>46055.48997685185</v>
+        <v>46056.3003587963</v>
       </c>
     </row>
     <row r="23">
@@ -1163,24 +1163,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Health and Safety at Scale - Logistics Business</t>
+          <t>Andre Gray is a Valiant! - Port Vale Football Club</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:15:24 GMT</t>
+          <t>Mon, 02 Feb 2026 19:18:57 GMT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQZVY5dHhMNlBKYnlkVmRxV1RlZ3hfdDV3T0FzQ1lTajZjaDAtSVV2RVlleUYxZWIxUDR2dXFhSEFtS1VGVy0yTnJQNVgtOERlNTJoWm5fVkFoaVJVajZiVXFhdS1WOFV2bFZKVl9IYjJkWURkWkxyWmxrM3BTQll2aHpn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTFBmTTI3Q01qcGdCYjR1Qklwa3JNNTNNUlJ0c0VNeGhQMTdVVmVYbGg0aEgxT0x2VDdlcnNLOEYtMDg0THU4MHlCcmRObDNfcnhabjJBTXQzNFdqVm5wWnNfUA?oc=5</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>46055.46902777778</v>
+        <v>46055.80482638889</v>
       </c>
     </row>
     <row r="24">
@@ -1196,24 +1196,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>THIS WEEK: Russian sanctions, Ukrainian loan and US trade deal - EUobserver</t>
+          <t>MPC Capital and Morten Astrup roll out new shipping investment platform - Splash247</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:00:55 GMT</t>
+          <t>Tue, 03 Feb 2026 07:31:43 GMT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPZ0RuX1EzcDI4OVJDVTRMbmJMdTRuR3I0X3lDX1NYX3NBcUZDdEZIckxMMDhnYTNDMjhJM3A5UDE0UVpIUnV6clFYWkNOS1J5V3p2a1JkUGt6X19xWE5kZXcxeDB4QlZpNHBVRlJ2TTQ1Vmd2UF9qV1VybEhuME1HdnNMd0pNOVQ5cHlsV2hOUzVVVm9STGc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxPTE0wcTV6QlhtSEtqaHZWWHZhY0dHNS1BOUJjU0UtQXNLblQydVVycUxFT2xoLWhHb0Z1cDVTYnMySmNBVFhBUUtkdGJkWE1DUTlJUFJ1emgxSmZVai1MQ19XUWtpQXZ1LWNKQ2F2c0ZWblR6OENXOXdRSmdIZmtDTkQyR1NrM2QwLW1qM2o1bmlGYzZPSm5HcEFn?oc=5</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="1" t="n">
-        <v>46055.25063657408</v>
+        <v>46056.31369212963</v>
       </c>
     </row>
     <row r="25">
@@ -1229,24 +1229,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Net zero readiness in Hospitality, FMCG, Manufacturing, Logistics and Retail - theenergyst.com</t>
+          <t>Targeted sanctions in response to brutal repression of protests in Iran - Australian Minister for Foreign Affairs</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:46:56 GMT</t>
+          <t>Mon, 02 Feb 2026 18:53:57 GMT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxPcENJelBLS2dmNFotWm5CLVpnY2h1dFhPbTlGYkJNZlRVSnVhNHJBZDFNU3lOMVNxWDRHc2NSYVpzZENlcEJaclRYNTB4TGhSNEM3b2RKMlA3TWxtN3NtMzFKaTNxWVNHUlowaVBGaTFHWnpQTlRSLS1SLW5tdTVJYjV5WjFtQnRodlg1R2V5dnNMWTJnNWlqT1o2al9pVUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixwFBVV95cUxQNF8xXzhtOG5yYXRXYk9Ydm9WSEdfd3NibzRuSmdtS2ozWFAycldxWHlNWVNoV29MTU94T0RuOVdYaHB1MXNDV3B2R1RfVXc0Y0tjc0xYOWlpV2dNWWxaaGxFQ3dwN2VGci1UTVRMLXV1aXpmNGxpTklXNWp2UW0zdGNIX2h2eVJHeGJkakRjWFpHTm5YR1VsTXlOd3FiN0NZdmFtZG12djR4MWRvYnlhc0I1elhqbEI3QXNMazlMeU1MOTFhRXNz?oc=5</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>46055.44925925926</v>
+        <v>46055.78746527778</v>
       </c>
     </row>
     <row r="26">
@@ -1262,24 +1262,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lamb welfare measures will be an “added cost” to supply chain, says NFU - Meat Management</t>
+          <t>AD Ports Group to help develop multi-purpose terminal in DR Congo - Baird Maritime</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:56:09 GMT</t>
+          <t>Tue, 03 Feb 2026 05:16:42 GMT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxNYUVBWXIzNWlWWGRsbk1lVXE2RnVqMEtNbG9KR0YzbWlVTGJJNnpDaFN3YnRzMExRZlBESGxRem9mSXkxSEgySVpsSkxqM3pLSDFjNHdnckNmN2JtRGxFUWJYVTNYci00ZFdHbnE0bU5ZYUNVMmNGOEgxelc3cDJ4bXBVOGJGMlhOUlVhcGFWTkxLZjFUZU9wT2hOdk16Sl9XSmtpTkZYeXN6S0hDMVhSQzJrbW8?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQMzZZT0Z3ejBobWptOGdwTG9CemNtNFdyaDA5dkVEX0NXb0NhTzNFa0FYdUV5QjdjM1pyaXFtZGZOR0VnOFViR0hiazZSZUcycFIwYkxTUGxkU29DTkxXV1VrYmVYWUpIN3JTTlhZT0hqbDlUZ1l2ZHpzTzVwSjRmTE1mNHgyb3F4SG5tYjNPUERsRFBRSk5xbHRBWmpQNzdCdmJFQnZicnlUdEFJWGVr0gG8AUFVX3lxTE9OS0VYNnhRUHFXQmFkTmtLNUdIaW1RNlJKVmpLbzhxV0hqNXJfQmgwY1VjSVBDZnhWSUFOdDZoTHNUT0xqQW9vWWhVX05hLTI1NXNCbXoyN2Q3OVZtRFdNMjNQVkFkTlpJUTlwUHJyM2NxS2hSVFVqTTdGemtYb1RGc0dnT2NoSUVkZnlBRU15bF9mR0t3N0JDbnpJUE14U1p4ZG43bFpvQVhMcTQ2N25rQVhyY2VkTkYzYzY0?oc=5</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>46055.49732638889</v>
+        <v>46056.21993055556</v>
       </c>
     </row>
     <row r="27">
@@ -1295,24 +1295,24 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>The Compliance Inflection Point: Why Mid-Market US Insurers Are Feeling the Strain - Insurance Edge</t>
+          <t>The Clean Energy Supply Chain Europe Still Doesn't Control - Crude Oil Prices Today | OilPrice.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:02:57 GMT</t>
+          <t>Mon, 02 Feb 2026 21:00:00 GMT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOemlwSW5xR0c5TXk5ZXJtak96NktuWmpaUFRYcDZKWl9XMlg3dmJPLVZwOFVWQ0VuNFFUSWVSMEViZjhOZEpWbTZieXNVWjVwUW9QTGpucmVfQ2xDck55NEhsSzFhc2ItbjNmQkYzdkh4UE0xV05QLVFjM3hvc3BfTUZ3OGZsc1huVmFDVnhVWUVqVWFUc3NRUHN1VVZtRUZlcFZBcW9yTk9XU0l1aDBqX1JkNWRBYnJweW91MQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxONWNkWW5kTzhjYW1mT0ZXcXUwdVQtNW1GVzRFWTNwT0ZydzJxdlZJNDR6MnBpLXIwVDg1ZWF4ZlhmVnh3TG5FTkZJeDFGTk9yY1ZCSndWNVlFdWp2RWNjbUQzRmxTbDVBanFqVjBabXZ0SnlJcGZWc3d5NkdEdFFnYXVhNE55Q2ZRaUt5em4tWk5Vbi01TjJHQTN1NFNhTVpMNF9rY0lKR0HSAa4BQVVfeXFMTkNsSGJ6T2dMWXRKYmQ4M2tYbXNNR3NsRjVCQnV5TWJQRzVINWQ5ajlPY3A1Z1paWlhCakpaQTBQa0tvYmNJN24yLVlfdDRpZGpPV1pTWklPb0IyOHN1RU5qNFowd1F0Um1peU40RnF3RnZGc05paGF0TDVKdkQwazNxeXRDNERWaXNlempoSERvand2TEZnbHV1VzB4LV9yMGQwYjVHY29hbm5qY2RR?oc=5</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>46055.37704861111</v>
+        <v>46055.875</v>
       </c>
     </row>
     <row r="28">
@@ -1328,24 +1328,24 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Verdion plans €69m Greater Copenhagen urban logistics facility - Green Street News</t>
+          <t>Global Mobility Lawyer: A Focus on Compliance Means Clients Often Miss the Strategic Risk - Fragomen</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 07:45:57 GMT</t>
+          <t>Mon, 02 Feb 2026 22:35:06 GMT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxOWU1GQkF6aWxiaWs2RjVoWTliVE9UcDRBOTE1aWJENE82amxXQXlmcTFpMERCUlUzckluZzA0N2paT09VeWhtVTU4YlpNZkticm8wWWs3UzZ1Q1BRcXA5bzVQd0tJRGJzVHUxdmdhMW4yOE5XNm1vclU3UUIydkkxdG11VDZmVnk3ak1ZZzNBdTNTeXBQTjhwcC1QMV9sMXJX?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOb2xYMHdGQWIyV092NjNUWUdCWWtUYzNxTmplb2RVT1FQOS0tQzloQ1RtQkZEOE1DYmN6VXBqUnU2MDMxbWlDRFI1T3h4Ynducmt4LXROdmpaTmZfMW1QcVc5TVdQOTBuc2QzRU1MV21QRmVCWFp5YlFPX0t4MEVvLTdmTUI3S3liUnFSc09uUnVtdk5IWUhkeERzQUhFZzVudWUtQ1RFZ285S0VrTVFybldjZ090Zk5sR0oxLWxxcnkyYlFISGc?oc=5</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>46055.32357638889</v>
+        <v>46055.94104166667</v>
       </c>
     </row>
     <row r="29">
@@ -1361,24 +1361,24 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Clarion Partners Europe acquires French logistics facility from Affinius - IPE Real Assets</t>
+          <t>Trump’s tariffs are keeping inflation from going lower, report finds - The Independent</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:33:47 GMT</t>
+          <t>Mon, 02 Feb 2026 17:29:00 GMT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOS1g5VWhPM2VtR3lQSC1sVFRDNmhEVl9IdzYzWUw5QS1sVXgxZHhWc2o0bkR2WUtNTnlsUm45VnZiUV9ZVnlIeGdWbW1jbXhOYzViQlRxSEZtaHJoODQ1ZW96NHFHSWJtUGNqZC1xM1NVWnk4clcyT2VQSVhaRUtWRjdUQnlfWnZLOXM2dlFyaFNtWUQyYndCcDZTWHZXVnFLNWlRdV81NFdfWnUxcHVzMm1lb005R0FsM2g4aFJB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPOE5VQ0ZELW0zcHZyQ2JYdzdOQWJ3ZzNheTB5Nm1FRHk4aHBOQ3BOWlhYOEhBSEo1Y09GYjRsM3hqWnA4dzh4Rlk4ZHM5cG9lcjVQeExack1mMTUwRW9GWDJfQW5EQk8xTkJQdHBXUnRySEdGckFWVG9XR3RhQWQySFlOVWZFcGxtdTh4NURHSFJwWmE4QzlKRXpqdEw2YktYT0MzcXlFc0I5NzdjdTFNSmxiNlZPUzQ5MVJ3NmhEbw?oc=5</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" s="1" t="n">
-        <v>46055.48179398148</v>
+        <v>46055.72847222222</v>
       </c>
     </row>
     <row r="30">
@@ -1394,24 +1394,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CEO of World’s Largest Container Shipping Company Says ‘No’ to Arctic Shipping - High North News</t>
+          <t>Asia’s SITC extends container ship order tally in China - Shipping Telegraph</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:50:10 GMT</t>
+          <t>Tue, 03 Feb 2026 02:01:12 GMT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQU1ZCNTRWdUhWN2VyUzZQbmlwSDFFNFlwckhWWVhMazdIR1lFQmhieUxBYjJzLWFUTmdsRkVXdFdndXlVWWtoSDNTUjFhUHBQMmQ0a2RVcVhwR0VmM0tpN1ZVTVlWNE5tV1RHVEZmdjNXa3JqQ3lRbmdOVnFGNndTM1FuX1lnU2p1alBuVTBxT1ppSmwtT2NUX1NETk1PVVN6M3dlSlFLNnMwdGVqWFU0elQxYWc4Z3lWVGVCQm9WQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxPdkd1NDR3ZnRtVXdmSDNSNDktd0F1aDM3d3lRZFdQWVVFcWtFS1lQTnZ0QjVJb3dFVkF1bHMxdnhKU1IydFVyMDQ3WFRURjgxZHNlZXljX0pkSGFNcklyZ3pGandDcnhWa0xwWDljWTg0SXpaOEphbnVjZjJLU09tc1VLaFViRFUyMnh1bkxxTmRwNVJTLXhDMFdRRGhWc0dfWVE?oc=5</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
       <c r="G30" s="1" t="n">
-        <v>46055.45150462963</v>
+        <v>46056.08416666667</v>
       </c>
     </row>
     <row r="31">
@@ -1427,24 +1427,24 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Skarv Shipping AS selects Oceanly Performance Plus to support automated data integration and digital fleet operations - shipmanagementinternational.com</t>
+          <t>Tariffs are reshaping Canadian manufacturing, but not all workers are being impacted the same way - The Conversation</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:34:37 GMT</t>
+          <t>Mon, 02 Feb 2026 19:08:28 GMT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxQM2RvOWNMZ0JQblZOSjV3NHN3eldnckFLNldOaVc2cmU2YXRvakdmM2NhSlFXVmpmVnN3MFdrUjJqMGJxaWlXZFM4YVBPY2xBeXVETmVJYm9aMFNJdklfNmlkclNSbjc4X1BxcGluM1NVel9PN3R5VGNQVWJYVWw5T3ZfbjdhQ0UzdFI4QjFOOUs1M0JfNkY5cXVFN2hCNExaMTVBZG5XaW1rQ29MUG5waGdfQUs2OTV3TE9wVmdBeXN1VTUxSnd6NnNPOXBwYlNJS1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOaldJdHBoSHA2cmtTcUNIVXpxWGlvZk9RMGFKNjBDS3RlQmtqRS11b3pUZjlVX2JiUTZnNkcxRHdzTHFkZF9oa0V5R1JjY3hSS3JqR0xrQU15ZE92SU9kbmp5X1ZESXJ4dFFWMFJyREkxOXJ2QUJFREtIYkxJVl9IZGJ6UE1WQm9obUxQbUxlUGYyQlF6U01yT0VkYVhELTYtT1p4TXBCWE1yMTJKWV9GTUVtajVhYWd4bFJ1UDBXTGw4cG4yRHA2a3dMUQ?oc=5</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>46055.44070601852</v>
+        <v>46055.79754629629</v>
       </c>
     </row>
     <row r="32">
@@ -1460,24 +1460,24 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Shipping investor J Lauritzen hires new head of research - Tradewinds News</t>
+          <t>What Is a Supply Chain Risk Management Framework? - Z2Data</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:03:44 GMT</t>
+          <t>Mon, 02 Feb 2026 20:01:15 GMT</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPNFZvNVlOdXhWeEVPakxtRTVVVkppb1ZmUjJmRW5mcGNsWkM3OWhpNW1IQldqVmx0VE9WSVlvc2N0TmloNDhHUUlQVlpPN1hzaGx0dkE2dmhqVURaNjU2U3ZyR1l5cnlfcHBCRVRzY0tiZEF1b2x1MjZQYXVDa25GdkVhZmhBOXEzUllVMHU5d0I5Ynl6WkJleWZQQ2ZjYUlhWk5qSHZTd2hRdWs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxNck5ocEx0V0ttWmJuV3VMel8xZE5DZFNONU0xbS1fYlpwQ2taa2NiTjZTdl80TkpWZzFBcXE5MjR5UTBTSFZGUnlIZmtmTFNyR0k4cjJCek9Nb1ZtdmNITnhzczY0Q180Qy0zTld3MHN3QUtYVjhUY3BocXJ4cUZaNk1jMUI?oc=5</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>1</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>46055.46092592592</v>
+        <v>46055.83420138889</v>
       </c>
     </row>
     <row r="33">
@@ -1493,24 +1493,24 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Abuja Pushes for a Modern Logistics Architecture - Air Cargo Week</t>
+          <t>Columbia selects Prevention at Sea as its compliance partner - Splash247</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:13:26 GMT</t>
+          <t>Tue, 03 Feb 2026 04:22:43 GMT</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1BZENaWFpKQldCdHo0UFpwTFZLdnBLYU5aZFc1TlhSaERkZGNrYVdXVk9KX0ppX0haX01lWUdRQjljV2pCVWFxamlnTmhpbWZTUGNyOGdRSUxWVTN4VlRUQXdYX3IxR2FIQkVrUHJoRzJQMXIxYTZNQTBwOV8wNGs?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOMXpnenB6VVpjMWltS3d5OGhIS2x0a25LYndtVzVHS2FzRmp6WG1mUkd4WVp5MFdVXzQ1MWpNUXBKcFNSZkQ2UTBDN1dGQUFQb1JudjcyOEtGMkNlaVJLVVd0eHNTRDdacHc1NUVHdlo0cHctejBYMXA5dm1YeHNHWTFXRjJKaFgtNnlJ?oc=5</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>46055.5093287037</v>
+        <v>46056.18244212963</v>
       </c>
     </row>
     <row r="34">
@@ -1526,24 +1526,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Panama Canal's new ports and pipeline tender processes begin - Seatrade Maritime News</t>
+          <t>Epstein helped Dubai businessman lobby Mandelson over £1.8bn British port deal - The Telegraph</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:18:55 GMT</t>
+          <t>Mon, 02 Feb 2026 18:07:00 GMT</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxOTC1BSEZJYVZRVk1qSTNOS3VGbDlnTmpRWnFCVkUxQ2FYYklBajIwVGhfaDZ0dHRaTXMxWEZtR0lGSG9qMXRYU0JjanF1dlZPQ1FHQ29hNkJHYU5fTFhqNE5iS1JFNGVKUTZCd1VURUk2NDRTZEluS045ZVlPdkhoX0w0RmJBZEpXTUFndHdwWW9HdHlTbEozVjJJM0pOV1ZFeVhIc005TGNWS1c0Nkdz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNT3RtdThCZHJ6TV9ydks0ZnFVRWE2elh1V0w5WU1zTm9oSWFZQU92bnJGQ1FZZTV4Ql9UMFVzbXZubnlGMVFIZHRmNk5LOVZYSUdmcGFKaFFDS25FZGtYOG1fLVVoeXdIb3kwMTdfV2RTNTVvY3lDcklqN2J3ODUwV0dCMmpCUHRrbWlxVWUxTm5XcDdJR0xNVVhtSGZZUQ?oc=5</t>
         </is>
       </c>
       <c r="F34" t="n">
         <v>1</v>
       </c>
       <c r="G34" s="1" t="n">
-        <v>46055.51313657407</v>
+        <v>46055.75486111111</v>
       </c>
     </row>
     <row r="35">
@@ -1559,24 +1559,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Norwegian court rules sanctions against Russian fishing firm Norebo are valid - SeafoodSource</t>
+          <t>Martin Sherif is a Valiant! - Port Vale Football Club</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:51:44 GMT</t>
+          <t>Mon, 02 Feb 2026 16:09:02 GMT</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQY3FfUTVqdHJrN0VGdXMtWjFmUE9UYWtLTzhabFlfLUw3OHRYMzlrZ1JOaWh6NC11LWxGSXk3QlZvb3lzVnBzNmlQVmdBNjZCeEsyeVV5VWNoUWR3dG5qNmNiNUFHeThrOEZkOUNtVGNEZjItTG1QT2xUN2VOYzJ0Vk1kQ2VpMGFqUF9DZTh6bUZhU1NzSVhTdkR4a3NNNFhEYkNEUnNPbW5nc3pvQ3FoRXRpd1lqQ3M1QXdIRUZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE9ydllkZXd6Tld2X0VoYlhjZEJtQUliTEhYQncyTVpBZXpsaU9FTEVyU3F2RllYSUxONFZyd0lzZFMtWHFHeHQ0c0NFTDItclJOYW5lT1VvYnJHMnlWeUNHRzZTdFU?oc=5</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
       <c r="G35" s="1" t="n">
-        <v>46055.45259259259</v>
+        <v>46055.67293981482</v>
       </c>
     </row>
     <row r="36">
@@ -1592,24 +1592,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>APMT open to temporary operation of Panama ports - porttechnology.org</t>
+          <t>Vale confirm first-ever Hall of Fame inductees - Port Vale Football Club</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:55:34 GMT</t>
+          <t>Mon, 02 Feb 2026 15:09:03 GMT</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPYWNPVU9TXzUtb21BS2tJdEZPUkhfNFR5T29XRXBaX3llTkhwYVpQNFZPY0w3YUQ5NDktdVdPajNyc1F1Q1c2QTFOc1lqSlZpZWs2c1N2YmpDU1lTT3ZUeENDWnVrcmxnaDI4SzM4NGNEMGdVQ2paV21jLXg2NHIyMzlEZkdSVzZLTUdLZmFR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQX2ZjaVBpdkF0aHlpTlhRcXQ1QWJLLWxiN0YzZEFmMmlEdHpuS181YzMyMk1KRjZpdXA1QzctclF0V2pMN2xvdTJTNElXcFJzQjNqeGFhb0lMdUdpRTBPSlpxOEdfU19xWWdkQUxzUFo5SDRvaGNyMzNRQUkzcm51OUZB?oc=5</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" s="1" t="n">
-        <v>46055.41358796296</v>
+        <v>46055.63128472222</v>
       </c>
     </row>
     <row r="37">
@@ -1625,90 +1625,90 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Transport NorthLink warns of seven days of disruption as freight sailings cancelled - Shetland News</t>
+          <t>Tanker stocks off to blazing start to 2026 as sanctions trade continues - Tradewinds News</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:31:32 GMT</t>
+          <t>Mon, 02 Feb 2026 19:16:41 GMT</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNTUJsLUljdDNSNEx4SEFZWTc4TEFkaFFMZzg1ZUlJVEkyMGt0bXNIamlZcXlzSXk3YWVBMkZSZW1Na3hHaWxkVnRCNHVvVmlfV3RndkdxSGswaVcxVV9waWxCVlBTZmFQMlRrZ3R6UkphZHpycUdMQWpQYUpFaVZUU1pR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxPb2lRMExjOXNsWFVhQU4ybGNoTXpOMS13WUE2MGxLVzd5Q0JqRGxLczBmbFpiOUJGSGxVZ2l3dGxzZXpHYlZjdVBRSE9Yak5tenh6ZE1MaDNFV1JLTlJMMHNNR0NCWUk1TUFGT0NkbjQxSlZqWlJBalJSS0JaUG4zaWFTYkQ3R3lPdWJKTWZGdE1INGxCc2VuSjhXZDhaclROTi1ubTRkSERHVWNXTGpkVVBnclpjZ0UxLTc0cDdFdw?oc=5</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>1</v>
       </c>
       <c r="G37" s="1" t="n">
-        <v>46055.39689814814</v>
+        <v>46055.80325231481</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Crystal International unveils advanced logistics hub in China - Just Style</t>
+          <t>Russia resumes strikes on freezing Ukrainian capital - The Times of Israel</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:57:30 GMT</t>
+          <t>Tue, 03 Feb 2026 05:08:37 GMT</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFBTLVJYX3pEcmhvNzAwR2tNVUZjQmJGbk54SVpwLVhxOGVrQ1A3NmtfY2NlTFY1Z0Jwdzd6QzhQN19QTnI5Y1h6N3RHUWZNczFDNlVCZXdaQVlSRXhsaTN5N0VSMjY3QUxtWWh3cDA1djRROVd2ME5nQWZjb2dUUVU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxNem9RZ0trLWpVZTdfQjVUS0s2eWRBOTg4djdzaHZWbGxSLUR2NGFmVm1EM0lkWWpXUl9GRkRobnVwSDVvTGIxa01PVEVrLWo1RVBsdUFFYnB1TDhwa1BvVDlPbXRUdnMwUXZrc01lQy1iMDBONWFvYWswT0FRZTd5ZHpsQ2pTczJ4cVl5UXBWSlpIVDZtMU1qX04yT3UyU1E?oc=5</t>
         </is>
       </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
       <c r="G38" s="1" t="n">
-        <v>46055.45659722222</v>
+        <v>46056.21431712963</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Supply_Chain</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>("supply chain" OR logistics OR shipping OR freight OR port OR tariffs OR sanctions OR embargoes OR reshoring OR nearshoring OR compliance OR "supply chain disruption" OR fragmentation OR instability) AND (company OR manufacturer OR factory OR supplier OR export OR import OR production)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Freightliner acquisition by CMA CGM completed - porttechnology.org</t>
+          <t>Iranian police detain four unspecified foreigners over unrest - Yahoo News UK</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:45:34 GMT</t>
+          <t>Mon, 02 Feb 2026 11:28:46 GMT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxONmpqaUtvSnJHMGhhWUlBQ1hXdjJ4V25yTUZGMElZQ0NmNGdUODBFYmE0NThjUnl3UG1lbEZ2RVcxRDVlV0hvcmxPS3F1dDlFZExSY25lUkIyejBJTlRvSjFVZmU4R21zTHRaamRIY0c2ZHdMdzJfM3pqQWpkYTNHdEdUdmtBOXJ2ZXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPekRjSmNra0R3WlRGV2hzZDRMWjNkWEJiNE9Jb1RfOWx2WG45cE15cGwxMXMzMm1FclVYeTlBeE1WQ2cyQkVVQ0kzSDkzUUR2TVhzM0psZEtyOUxVWUxhakllLXhEWXY2U2dJaDNmeF9pTWE0Z3pKMFJtaEhqOVJya0JIY0FBZw?oc=5</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
       <c r="G39" s="1" t="n">
-        <v>46055.44831018519</v>
+        <v>46055.47831018519</v>
       </c>
     </row>
     <row r="40">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Update after police called to convenience store - Cambs Times</t>
+          <t>Police statement as flag-waving protesters march on Hanley - Stoke-on-Trent Live</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:04:00 GMT</t>
+          <t>Mon, 02 Feb 2026 17:30:00 GMT</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxORnRnWW9xTkxDMVVISlZvNjZVS0RfZGhhLUU4RFBNZVNsbmExOEJZZHVBZ1IzelZXVl9nOGZFZGQwcTFfaE1YZjlUODVJWExsXzNiVm5DMnpQNGM4RHplZXZRZG5HMHNjaE1VY0VjOGdpd194cU1rUmMzQ3NXV0QyWXBoQkYzMEVVM1A2eFU3VlpkYTA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPT1otX0VCaWwyTFVjMkhPU0habVRyTlZTWl9mYzRJX1RvcUZoTTBFbmd2NENQNVJOcW5aajZkLVFRZlZpUVM2MERmUDFCOWp3bFdkX2lseWg3eHByak9HUmlnV29OSlViX1ByNnExQllBQXdXeHRzNU9hc3RlMEY0d3otTjhkTXc0czZ5QVpYckJhNHpCajV5NWJuNG15SEt5NkNuSGNwR23SAa4BQVVfeXFMT29GZ3RWV0xJczVuSG91dVpCS0dXREVJNG0wQUhkU21sYTY4MVItR2pocTdpMC1obWRKeENHNFdkazgyZnpVdzRvZFotcnRpb1lxWk4tbW1hdkxmZ2duTkUyTGcyN2pGWG5iRE9KclhHeVdUUzg0UVVyR1pha2lKdUlYMTViQmF4b1lfc0ZGMlVZNTdEU2NoQU5rb2N0M0p5dGZDVG1USzdCWXJhdmhn?oc=5</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>1</v>
       </c>
       <c r="G40" s="1" t="n">
-        <v>46055.46111111111</v>
+        <v>46055.72916666666</v>
       </c>
     </row>
     <row r="41">
@@ -1757,24 +1757,24 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Iranian police detain four unspecified foreigners over unrest - Reuters</t>
+          <t>Update after police called to convenience store - Cambs Times</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:29:03 GMT</t>
+          <t>Mon, 02 Feb 2026 11:04:00 GMT</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQbEFYWUliVTVUN0ZCdEdQYVNQQWl2VUJqakF3S19nbG1BMjE2M2xDa1NLRXI3U1pjVFRsWGZhRUFfMnQ5cjdPTmF3VFlpcENfenhkOTFWOXhMckdETkVINWNaY3RCMWxwTElDVzg0U2xLamVuSXlVQXJ0RmpNb25taUp1aEFJc19IRXdhZk9DZHE5OVQzSnR5LVM5QmdhZFNHT2dPY2ZvNDVPSlhTdVRLdjJZMldiZkZaTzFsSA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxORnRnWW9xTkxDMVVISlZvNjZVS0RfZGhhLUU4RFBNZVNsbmExOEJZZHVBZ1IzelZXVl9nOGZFZGQwcTFfaE1YZjlUODVJWExsXzNiVm5DMnpQNGM4RHplZXZRZG5HMHNjaE1VY0VjOGdpd194cU1rUmMzQ3NXV0QyWXBoQkYzMEVVM1A2eFU3VlpkYTA?oc=5</t>
         </is>
       </c>
       <c r="F41" t="n">
         <v>1</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>46055.47850694445</v>
+        <v>46055.46111111111</v>
       </c>
     </row>
     <row r="42">
@@ -1790,24 +1790,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Another e-scooter taken into police possession - Fenland Citizen</t>
+          <t>Ukraine's capital of Kyiv, other cities under Russian attack, officials say - Reuters</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:33:00 GMT</t>
+          <t>Mon, 02 Feb 2026 23:23:20 GMT</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQY0xxNnhKTTZwdUtJdVZNZXBSQ0lwUlpxMDhCUWxhUFBFLXpUaDJMNmF2OW1YY2hWSTJ5Zm1Vbk9mcDl5UjZpWm1Jd1FPYW1mVk5sZV9xc3dlYktqRWlOQTFaUDBBU0JGMVhQZnRkSkMwYV9QWnpsY0RQU1VtRlhWWnJDb0o5WkIyWlZNcTVoTHZvM25keS1BRg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNVlBuNklvRHU5MVg4THZMa2VRMmlRZVpEb2FmX0pNNlJCNXNHbS1CWW5NaG5pbUNLZG05ZDlhcHgwQUV4Tm1mbXVuV2cyaXp5ZGZyNnJkeEJPdC0xR0NYYU8tOWVTX3NXSmNPUHhWSEg2dWlDZEFEYWhCOGdPdWFsMlM1SXYxU1Q1NlhTcFRfLVB0SDM4OGRYVDQxNVNpd0g3?oc=5</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
       <c r="G42" s="1" t="n">
-        <v>46055.48125</v>
+        <v>46055.97453703704</v>
       </c>
     </row>
     <row r="43">
@@ -1823,24 +1823,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Police probe launched after jewellery thieves strike at vulnerable Smethwick woman's home - Express &amp; Star</t>
+          <t>Police Urge NLC To Shelve Tuesday’s FCT Protest Over Security Concerns, Rights Group Pushes Back - Arise News</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:11:04 GMT</t>
+          <t>Tue, 03 Feb 2026 06:13:14 GMT</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxNSGdYOGR4YWRSQ0pFc0VxSUdoc3RNUkZ3bXRvdDBuVDBBWWhYLS0td1lPVmtDUWYwZGpqbVZ5RkxrMWQ4SkRqWHhBSkFjWll4QU11cnZKMEtRWTRmNi1xOWRsWTlnSmtkSXN6MVZRT2hCZHBnR2dlbmV1NzZBcWJ5SnJZcDJWNWtENVFkdVNKa2wyRTFkLVJRWDJTSHg2MlZUUDNWY0xOcFBuTkpWUUdRZG0xZzkyeGstTkdVMHF0UGo0UVlzYmNfdGQzMFVKNUtvMHF3UlpRSmJhR211YWFJQTdZVFFXSDJRU1lWNXQwQmxFQjNFMHk0VnFB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxPdkNxV2FzejFFR0dsLTNlU0JSMDRocE4wZ2hyNzU5dGVuSnd6M3JOQ0lLSkZWYloxXzFub2VGcjFJcjFscWZxSHlRRXJTdkF6RmJjell2T1ItQk1CQTlFRzZiMGFhYTRYV3dIUWFKV3FpcFNJNXEzT0lWUjVrc0hwZHhLeVVYTHRVZmdXZWdGOWc5YmgyemdRNGRoZWhlbDZuS19rZlZNY1oxcmxYQXJQX2VYdVFGazA?oc=5</t>
         </is>
       </c>
       <c r="F43" t="n">
         <v>1</v>
       </c>
       <c r="G43" s="1" t="n">
-        <v>46055.34101851852</v>
+        <v>46056.25918981482</v>
       </c>
     </row>
     <row r="44">
@@ -1856,24 +1856,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Police and crime commissioner storms out of hearing after being censured for joining anti-migrant protests in Crowborough - GB News</t>
+          <t>Spokane police chief apologizes for officers wearing masks at protest - The Spokesman-Review</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 15:14:07 GMT</t>
+          <t>Tue, 03 Feb 2026 05:50:11 GMT</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxPNzRfSWt4cFdoY3NpZmJoN3JicjVvcThEaHRCWTdtZW9CUWxNOEVNMURnV05DQ2hGUmJlbUwzbTg1OVZBTkJJaHBZc3dRMUNqTm5rQXBQeDQyMWFIQnh5bHJNWURBeTBJd1Q3OWJzMmNNeVZtbFg4NnZlX0QzQVRNZTdxUThmcjZONG4yaUU0SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOZHRHU2VfME5sVTVoQkpLMmpoVUhPN1lnZzdCSm44cVRfZ3k2NFNIVVdMSTh3cXIwU0RFUFNfZ1NMdXhrR0FXVEx0NXNadWsxWEp5WVU4cHBoNkgzV09GcEVtSEpwcG1jdkZWR2h4bjd6QWhfQTRtazA4ck14VXFvaVBDcmlKdDJSVHk0TkZacW5XTTFjQ1dMYmI1Y3VoQQ?oc=5</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
       <c r="G44" s="1" t="n">
-        <v>46054.63480324074</v>
+        <v>46056.24318287037</v>
       </c>
     </row>
     <row r="45">
@@ -1889,24 +1889,24 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Eight Arrests made at Demonstration, including Three for Assaulting Police, Queen Street West and Bay Street area (Mahnoor Mohyuddin, Jennifer Vong, Kyle Stephens, Woodrow Fraser-Boychuk, Abe Berglas, Darcy Belanger, Bryn Williams &amp; Charles Kaake - Reddit</t>
+          <t>Another e-scooter taken into police possession - Fenland Citizen</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:33:10 GMT</t>
+          <t>Mon, 02 Feb 2026 11:33:00 GMT</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPYlA1UmFxRnlZNXpJODk5X0hOWldUOElDdG1mVXhndl93LUhackpTa1FYZDBjRWR1dmFhc2xrYXMzMFo4WV94OEtZb0ZpYTljNlJYb0RVd1llS0RuWmRHRlA4QUFJaG5QTzBzaDRKUFBBUWNDR1pDdklZUXBvdnVqMmJiMVZydUp1Q0hVV2IydDZQY0F6eGtYdXB1M0w5QU8weWVEag?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQY0xxNnhKTTZwdUtJdVZNZXBSQ0lwUlpxMDhCUWxhUFBFLXpUaDJMNmF2OW1YY2hWSTJ5Zm1Vbk9mcDl5UjZpWm1Jd1FPYW1mVk5sZV9xc3dlYktqRWlOQTFaUDBBU0JGMVhQZnRkSkMwYV9QWnpsY0RQU1VtRlhWWnJDb0o5WkIyWlZNcTVoTHZvM25keS1BRg?oc=5</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>1</v>
       </c>
       <c r="G45" s="1" t="n">
-        <v>46055.52303240741</v>
+        <v>46055.48125</v>
       </c>
     </row>
     <row r="46">
@@ -1922,24 +1922,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Clime Capital Announces March Quarter Dividend Guidance Of 1.35 AU Cents Per Share - TradingView</t>
+          <t>Hungary Raises Alarm after Slovak Police Arrest Politician over Beneš Decrees - Hungarian Conservative</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 01:59:00 GMT</t>
+          <t>Mon, 02 Feb 2026 14:09:31 GMT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi5wFBVV95cUxPaERFNTN6UzRGZkxwdHJpTzVWdm0yOEgzM083aFUwVnZXbEpYbFg2cTFndjF5a2xSX1lFdzBkb3h1TGhIODRfcWh6dUIxdnJJbTFURTQ5dnJxVjFOVHhoZk41dHlrd1VDMi00VWpuSURqaWVQYVBZTHhrV1BFMVBnMkM4NEJVNExLenEycGUwYVBMU0ZldGE3Z2x3SGd2UUtOLXJDX01VYmpJYmNDMTJBcmNuWk9GUnphbHRranNOWWVfbGd1VlZBb1U4cWFmRXJVQWpWdDBEQXd2RVFrN2pTbTNhU2NXXzA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOSGNwRENjNUNNeDMxSWhEWndpNk9OQnpBV0EzazV3b1FSbzlic1lTUTFxTDQyY19UckVZYzB2cy0yZUhYNFF0dHJ1WEtXRDNSQ2VjY1B5WXZiNVA0UEJNLUo1SmxScmhEYS1NQUtoX1pFWjU5dUdqeXg1d3EycFZTZFFkSDlsRFptSHQ4X2lBenowTnZMNmtwRHh3bGQ4ODdzTlVRRzZEeE91ZUl6M2lFSDZoZ2Y?oc=5</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>1</v>
       </c>
       <c r="G46" s="1" t="n">
-        <v>46055.08263888889</v>
+        <v>46055.58994212963</v>
       </c>
     </row>
     <row r="47">
@@ -1955,24 +1955,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Police Urges NLC To Cancel Tuesday’s Planned Solidarity Protest - TVC News</t>
+          <t>NSW protest restrictions extended ahead of Israel president's visit - Australian Broadcasting Corporation</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:51:00 GMT</t>
+          <t>Tue, 03 Feb 2026 03:21:47 GMT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQUzc5Q3FUNzJteVlSUEJQekViSS1GRnJ6NFlmd3NVTXRmRzhCVWJfVXNsMk5ENjQ4MDJoOHR0MXZYSzZHbGdQTXlQVGR1dkU1eklxS2wwZFBXbkVybEV2cTl4LVRPNkFXdjE2Z1lySDJEdWdIX0lybnp3R2s5VjlzQkJQVmhubjQxMDBnMmhaUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOR25CYWQ2V3BfQnRxMmVBSEFDY1RzSzdhaThTcVU0RWdLX0Zyc3IyS19yck1YZHhiQ3R1OVdkc195bzYtR0V5UXlLb2Fta1JkaldFOU9QYjJpajFrczNQWHBTeGZQRi1jMXIxcXA2Ql9BQm5jOUVyZ2ZxcktENTBoY010OXcwZ3VjRXZ2TXIybVJ1dHZBT21NdlVSMW9Ea3RjQ3UzcUpMWTNxQUZEQXc?oc=5</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
       <c r="G47" s="1" t="n">
-        <v>46055.53541666667</v>
+        <v>46056.14012731481</v>
       </c>
     </row>
     <row r="48">
@@ -1988,288 +1988,288 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Clashes in Turin Injure Over 100 Police During Social Center Eviction Protest - mezha.net</t>
+          <t>Reno police confirm battery report, citations after anti-ICE protests - Reno Gazette Journal</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 01:44:25 GMT</t>
+          <t>Tue, 03 Feb 2026 00:14:00 GMT</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxOSVlDdkdjV3ItWWNVWENjVFlDcjFZb19jREVfb1FHVUtvTGZyeHdMY3l5WkMtVFI1MjlCNS13VnNidksxdU0xSk9sRUFwU0IzeTJVRTRmLVBFeXgzZGNsMEhnNTgtb00zUnp3eDVkRWN5aTFMVU4xMTZlUDNMd0d3OU5sNUpXMFRpamhhY2NVOGpmT1M1NEtMcDdlNWwwdHNYNGs2MWJsRFlSd9IBrwFBVV95cUxPa2NMbGltVmNON1BvS1lQMnZ3cFFzWFVtT240Vnl4QkhiN2UwUFhkTGp1Z1ZpRHRkTlhOZjdaVTg5MElzbjV1d1FlYnV6Ym92RG5YMHFja2p6WjFXVzNzb2EtanVmcS1rTUlWcS1peWRfS3dMWjN0ZTdrMWxBX0FDU2tfWWc4bzFjWVFFZXl2cUlOdUV6ZjNfNkZoOEswc1h2UzR6S1RDVUU1WDdjWEtB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxOYVFWYkdQSUEwVkstQUVseXZ5TV9uTGtqbFFadjRwcXozcWJfaF9GQ2xsUXZHdXFyaVVFMXNmYnhUR05PbFJLa3UzN0lVUEIyX0J5RWM5VlRLR2VpRE5raGdMSE5DaFlaZW92blRuZEl5WUlEQW1aZW4zUE1CY0t5ekY4NlFuazU0cHFTSjN0bTlwT3p1Z29vbTJfcTB3R0p0THliSzNPN0NQODdoZGgtMHY4d25vUUNST1pSM0tPTQ?oc=5</t>
         </is>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" s="1" t="n">
-        <v>46055.07251157407</v>
+        <v>46056.00972222222</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dow to replace 4,500 jobs with automation and AI as shares decline - Packaging Europe</t>
+          <t>“Everyone Stick Together": Eugene Mayor Kaarin Knudson on Protest and Community - NPR for Oregonians</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:08:32 GMT</t>
+          <t>Mon, 02 Feb 2026 22:40:00 GMT</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPUG85LWpVTTB1ajhzU3dMMEtCa3NkMDRxbmpjZTV4RmlvZ1dpSlh2VmZZSW40VEV2QzcwTDVaQVltdnpKT0gya19GT3I1VnJFUGNjRkNGNUtobGFCS0RjV2x1NmV5YTQ3bzlYUWxHRl81dnpLVk1vVHlEemtUU0JDeDk0SVhDYXBsSG9pMXBJdnJfOWpPQ3U4NjNVWm1IeEhCT1l6aWUxQ09EaGg0czl5MXh3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi0wFBVV95cUxPaDRwdTVIc2RfTE1LVXJLanlzbjFxTFlHVzBlY3BFaXZRRF8xQWJySFQ2eG9TV0s4b19MOFNZNlhvTTZTMDBMSlF6SmdvOENVTDN0NDRIbFk5R0s4ZGlQSEhvNHlObFN3Sm1MY0t5UHFudzNpSEV4TFpWblNZWEhmU2xwRG8xWHVRU0xDZTRFbFB4V1hfdncxVmlNM1VxcW5QOTI0Q0hPeGpOYXlwUUZtYlFpOGdLcFVWOUk1ODI2a1FRX2w3OTFKTzR2OUEyX0lsQlpN?oc=5</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>1</v>
       </c>
       <c r="G49" s="1" t="n">
-        <v>46055.46425925926</v>
+        <v>46055.94444444445</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Technology and human rights - Amnesty International UK</t>
+          <t>Ferndale Police answer questions regarding Friday student protest march - Whatcom News</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:19:47 GMT</t>
+          <t>Tue, 03 Feb 2026 00:17:16 GMT</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxPNHlIOVVoNVd4VmE2V3B1b0JLemxfMTcyYXQxakg2Q0dLekxWLW1nS3Myb3BnNk1TUm9Va1BzR3dSdE93SlRmV2gxN1ZoNmFKSm1YSGF3NUVQOG5qMi1mdnp4WHVBeXJ1MTlrWE42ZkhCaHp1cmhXQlMwMkd4czhaczJXWmxMT0Raa1JKbjhSZy1uUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPbzk1cHEtbWI4VjhaVXBCSXA2Y3MtaEhZWXAxYk0zMkl5SUVvcmh3d2JycHRiMTh1dEZrdGRqVDhwR0Z3UjJoX0JhSE1kUk9MVkVEbzZqUl9OcWY0N0ZRZFdJQ2FUQUFrWFhxUVk4clNFV2o4R0dMa1JBaVpFVjdyVDFraVBEbkR5TFc3VmZUQmNxazNhNlZiSGI5RTZnWnN2TVVGWk9zQQ?oc=5</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>1</v>
       </c>
       <c r="G50" s="1" t="n">
-        <v>46055.43040509259</v>
+        <v>46056.01199074074</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>The Telecoms.com Podcast: Ericsson, AI and Nokia - Telecoms</t>
+          <t>Police probe launched after jewellery thieves strike at vulnerable Smethwick woman's home - Express &amp; Star</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:28:13 GMT</t>
+          <t>Mon, 02 Feb 2026 08:11:04 GMT</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPTHhsYVpnTHdHNkNEQXR5YTVXeEdDSFh2dE9YLTJsdVdFbDV6MkxuQzJ5Q0xTdEZFb2VaMjlESi1JZDU1QWJpekR4ZExxY196ekhkZ2lJUDZzMnp5MjFrS250eDh5OGRSckRLczFKdjJKYVcyQlhmdEtSWTA2R0VLTTZUa1dhV2dlYXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi-gFBVV95cUxNSGdYOGR4YWRSQ0pFc0VxSUdoc3RNUkZ3bXRvdDBuVDBBWWhYLS0td1lPVmtDUWYwZGpqbVZ5RkxrMWQ4SkRqWHhBSkFjWll4QU11cnZKMEtRWTRmNi1xOWRsWTlnSmtkSXN6MVZRT2hCZHBnR2dlbmV1NzZBcWJ5SnJZcDJWNWtENVFkdVNKa2wyRTFkLVJRWDJTSHg2MlZUUDNWY0xOcFBuTkpWUUdRZG0xZzkyeGstTkdVMHF0UGo0UVlzYmNfdGQzMFVKNUtvMHF3UlpRSmJhR211YWFJQTdZVFFXSDJRU1lWNXQwQmxFQjNFMHk0VnFB?oc=5</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
       <c r="G51" s="1" t="n">
-        <v>46055.5195949074</v>
+        <v>46055.34101851852</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NHS trials AI and robotics to speed up lung cancer diagnosis - UKAuthority</t>
+          <t>Alderpeople Say COPA Should Investigate Chicago Police Conduct During Immigration Raids, Protests - WTTW</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:01:03 GMT</t>
+          <t>Tue, 03 Feb 2026 01:02:00 GMT</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNVW9sb25UeG1CVzdNOGVXWFRsT1ZBYWhwYkVTYkRZT0E3SURaNHdxeko1ejh5S2xnQThQaWp3TjRrOHM1TE1GcmxXcWFvMWZleFpRZVRNeWpQZW9fZXdBOVZjZTVJTjlUb01YTkRsZWZEQmdheTJ5d2ItdUt4b0JPX3RvZGZWc2JWZU5NRjVSbzNzQlF1Q0JabXRtemtYQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPN2xkVWx4dWpnd25XYVhTLXF3cXRJOGRSUDZIMFJaTGRpa3dEeVEzOUdKSzA4ajZWVk95XzF1aS1WdFlBT3ZVR3lBaTZMZDE2U0pvZWlON2xNZ0taeWxnTlJNU0NDdkdabUxyVGZnS0JZTk1KcG0xMkhVWU5QWWZqMXpWRkJGT1R1WENRZWpvMkNJV09RUlM1NjdhQmV3VnhOUkNrTE55Y2U4NS10ZGNSel9MbFlwUHYxd0lkMw?oc=5</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
       <c r="G52" s="1" t="n">
-        <v>46055.3340625</v>
+        <v>46056.04305555556</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Why banks shouldn’t wait for AI to fix the Gen problem - Retail Banker International</t>
+          <t>‘Significant animosity’ to Israeli president prompts further protest ban - AFR</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:28:04 GMT</t>
+          <t>Tue, 03 Feb 2026 04:31:00 GMT</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPNkJaSEM4djg2STlSalNWM0c3MmhmS1ZNS1c5MG14VUREZzNha25fVXp3VXF0YUczMkRlMEwtVldORHU4TFA1dEtLY3dfeXpmcW5UbHJLR09mX3FYZlFwbmtCbU1GZ3lsMFBUZmhpU2ZHMzlVZUxkSG0wNkRCeFcwQkk1OW5ZUlVaNXFPVktQb1g0djI5ZkQzU0ZKTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxOM3VBTUx1czNTbG5CVmlqcnF4bk13aWpUbnIySGRLbmZiSEtWUnE3RU1LVG5HcTJuSE1fVEJsSTVkNm5XemVYQjVwbk1TZWFKcGtYTVJRVUg4WkhhSzlqX2dqMFhjZXJ4N3hQQnAtdEVXQUlzTlNfdnVQZEVOeTRlUkJmMWFtVGxxajU2WGtEdTFFTmFuWWJwb1NxaDhWZElhYXVQZVdJSEhRbHJGeTdGNm1nb0FGZw?oc=5</t>
         </is>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>46055.39449074074</v>
+        <v>46056.18819444445</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>AI and tech adoption in treasury - Private Funds CFO</t>
+          <t>Police extend Sydney protest ban again in city’s east - dailytelegraph.com.au</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 02:00:49 GMT</t>
+          <t>Tue, 03 Feb 2026 03:01:48 GMT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE9HX2wxTWg4OXVDNHpST0Z0MGZsRVJZVkVRSHJyWVJKMmk2QVN1Rk9LQmdfSjF1a0h1Vy1tSEpyREJpajlEcWRjZFdYRlZiT1ltYk0wb3hHUm1GejByQ183dTJWMlFXQmVOdDdyVGpjU2lVOFU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxNUkkyMUZaR29JbkkxOGZHSFF1YmRFYUxNYU5RVENDbHhmU2h2anF3bzAxVFhDc1AwRGFTVDluWVJvNEI1QnViR05GTU1YOS1JbzhQS3ZOUGJicFpmR3J5WlBwM0VDbVZlUGwxc0NqNkx3YnNVaGFvaWlpcFBXN2dibi1YMGJJQkpHbmNMWl9tWmNSMzFPdkVZY0pwOFdlcFFDZG1aMDB0ejNiN0dNenVUM2FKZ2F5a2E2UU5CNl9tdEtiWmt2cnU5N3RBbktEelRoaHBhUnNrdUtUYWdMcEw1NUZsYWgwRXM0WnUycksyYnhSbjDSAfgBQVVfeXFMTkNJUVUxVkp6UXFlZzcwVTVmYUl2RVUwZVc1NTM1ZU9XeHVBXzRFNG4zTFZTZHZnWThnQWViWkd0WlgzZXVkMlhGZ21NVHZWb0JyWnU2TUpDZHNLeDIyX0kxa2VIMmJIQlI3ZGNVQjE0c3pLYWJobTV4Q1lCS3hxaVRUR2FsanZ2M2V6azNydDV3Ym5KdXQyZFNuY3NDRjhkQXV0VUk3djBkbmx6YWg4eEhQb3lzTHZYVDVtM2JiRDVfR0RaMlRPVEJsZnVTRjVmNlo0U3NOSU5VaEtOZ2RXUnFaSjlKLWpabXpmSDl0SHlUcDlvVEdCNW8?oc=5</t>
         </is>
       </c>
       <c r="F54" t="n">
         <v>1</v>
       </c>
       <c r="G54" s="1" t="n">
-        <v>46055.08390046296</v>
+        <v>46056.12625</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>IFR position paper on AI in robotics released - International Federation of Robotics</t>
+          <t>Eight Arrests made at Demonstration, including Three for Assaulting Police, Queen Street West and Bay Street area (Mahnoor Mohyuddin, Jennifer Vong, Kyle Stephens, Woodrow Fraser-Boychuk, Abe Berglas, Darcy Belanger, Bryn Williams &amp; Charles Kaake - Reddit</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:50:47 GMT</t>
+          <t>Mon, 02 Feb 2026 12:33:10 GMT</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1uM2Vnek8zdm5IV1hWem9CYWl1S0czMEJLd3lhNHNlLURxajlQZy1ISzdSd28yblRfeUpKV3ZsYWlPYlJsNGdDalFWMUQyOTVqSmQxMzNqV1Y2SE9UbzRxcjc3RzVRcTc0NG9tYV9JbU5fWVAzemRVMTVhV1o?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxPYlA1UmFxRnlZNXpJODk5X0hOWldUOElDdG1mVXhndl93LUhackpTa1FYZDBjRWR1dmFhc2xrYXMzMFo4WV94OEtZb0ZpYTljNlJYb0RVd1llS0RuWmRHRlA4QUFJaG5QTzBzaDRKUFBBUWNDR1pDdklZUXBvdnVqMmJiMVZydUp1Q0hVV2IydDZQY0F6eGtYdXB1M0w5QU8weWVEag?oc=5</t>
         </is>
       </c>
       <c r="F55" t="n">
         <v>1</v>
       </c>
       <c r="G55" s="1" t="n">
-        <v>46055.4102662037</v>
+        <v>46055.52303240741</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Protest</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+          <t>(protest OR protests OR demonstration OR demonstrations OR unrest OR "civil resistance" OR "civil disobedience" OR boycott OR boycotts OR march OR marches OR strike OR strikes) AND (police OR capital OR city OR arrests OR arrested OR union OR workers OR students OR rally OR tactics OR targets OR groups)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>How sustainable funds are navigating AI, defence and financials - Trustnet</t>
+          <t>ATN International Board Calls March EGM to Consider Capital Reduction - TipRanks</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:01:33 GMT</t>
+          <t>Mon, 02 Feb 2026 18:07:35 GMT</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPRktGQTJJdXpHeldsX3E3NEl3ckx2QjkxU2tIb3lPUF84dEI0a2ZfQjVjbTNMeHpZUFZjdkR2bldWTnpMRmNjMnBkNFZ5Rk05dW5xeEpsTWo1YkRXUjhpYkdEYS1od0dPSmhScjZPRjZsYVBxTzlUbXh1QlVrbVhwaFRyNTB4aEk4V2I3b1dhV1J4VC1vRUdsMmdTUEFFeElqbE1J?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNSEh4dktnUVA3TF9rTkJIUXZ2cFFkN3puZWpIN2dYTU9kRmtiRmtGUGFNWS1ieS1XQVc1QlJCcTdWZmx6U0RLRVhJU1hybXlDSTN5dkU5VmUtMVJKcFVYanF5WEdtUlN5Yk1USUhpYVp5eVA2M3MydWtKdHhwcV9FY2lSQUVueGRkaWRTNFYxemIxZkY3bnRBVlpzZTVoTUJPcUN6R1hoc1d5dkxzNE5NbzJaWjF6Qm5hTlEzQ2xn?oc=5</t>
         </is>
       </c>
       <c r="F56" t="n">
         <v>1</v>
       </c>
       <c r="G56" s="1" t="n">
-        <v>46055.45940972222</v>
+        <v>46055.75526620371</v>
       </c>
     </row>
     <row r="57">
@@ -2285,24 +2285,24 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Vera van der Burg puts AI and ceramics into "reflective" feedback loop - Dezeen</t>
+          <t>Technology and AI - Freeths</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:00:00 GMT</t>
+          <t>Tue, 03 Feb 2026 07:37:01 GMT</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiSEFVX3lxTE5RNF82VUc5cDNNTzhsdHpwbXB6TDBhNW80M2k2Y0NRbFlRYzdoV21GTDNEcko5UDdjbmxIVkgyeHhNWkRCLVJ0SQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBWa1dVRGdpcEZHemc2aURfM0tWNDlnRXJBRTRNa0F3Z25xMENnNHFmWC1henR2SkNXdnVYZ2VHa0lIcGo3UDFJb1hUWnI2R1c4ZDlpWkFIQlNPaGJBZTNGZUF4S2xnRl9qdG9wNGpGMV90aVpXdGc?oc=5</t>
         </is>
       </c>
       <c r="F57" t="n">
         <v>1</v>
       </c>
       <c r="G57" s="1" t="n">
-        <v>46055.375</v>
+        <v>46056.31737268518</v>
       </c>
     </row>
     <row r="58">
@@ -2318,24 +2318,24 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>AI 'slop' is transforming social media - and there's a backlash - BBC</t>
+          <t>CURE-ND brings together experts in AI and machine learning - UK DRI</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:54:06 GMT</t>
+          <t>Mon, 02 Feb 2026 13:45:51 GMT</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9wNDA2bFFUbmx5aDlVcjdxaWE1c1JHZDZTcmxnampFRW5PN19EejRhQklPMkJmeDNYZnlMczE3MWl0M0h2UkhpZUN5b0hoX0RRZzExcTBZUmV3d9IBX0FVX3lxTE9LZjR2U0dKMjJ1WktUTy1JaWFWUkluMWYtSmJBQ0J4QmVuTVhhTUZTUGN5eUZ5UDdGMFZLeHN2TWNPaHZPSGk4LUtlYkpuYVA1Vk9Gd0p3RThuWTNrYXM4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQQUxpOEJSX3VYSW04MTVNYkd1TnJJMXJKUjc2eEpZQ1I3M0hsSTA0dEdaWEc4dUpGQUpvYjRqbFM3akdkZHdzZlhpdmhhcnQ2VnpWb2otYjZjeF9JZ0h3ZTY0SjhDOTBrMVhJVTVXNUQtREczX2xMejB1Q0JKRDNkamFfSGVZMGp2U2t3N3VEaEFZaU1XR2xhQzFYY3RlT3B0OVhZX3RESzI4ZTQyVDZ6T1FxMHZiUQ?oc=5</t>
         </is>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" s="1" t="n">
-        <v>46055.28756944444</v>
+        <v>46055.57350694444</v>
       </c>
     </row>
     <row r="59">
@@ -2351,24 +2351,24 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>“A cloud-enabled, digitally resilient Europe transforms the protection of its citizens, infrastructure and strategic interests” - Thales Group</t>
+          <t>Alphabet Q4 2025 earnings preview: cloud and AI to sustain valuation - ig.com</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:08:42 GMT</t>
+          <t>Tue, 03 Feb 2026 05:21:31 GMT</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQc3lvdXNHRWx4aTVFNFlPbGUyTjB5UlVaN3dhSUhvbXQ5dmF1Tk91REd1QTU4R2VPbGc0b0VEbTZrRlE0cHJWaXVFYmlXaDFDMDhqM3BUOWtNZzJLb0FBSEh3T2pwLWEyTE5ycEpEX19mSmJ4TG40UTIzRVdZTk1IdEpFaWpfVmtoZFRTaXRBREk1YzdNdk1NOVJFRHpzdTJPemlFYmZiWGtuWEJJWVgyaVlDSDBsRjFoaVVUU2tjLU9ZUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQcnY4a2J0bWRPZnJxSGRHeVYtc05FaUY1MXgzQ3NEVkNJYjVIM1BCT0lFblVJN0xkUi1jZ0ZMQTZnQS1IYVB5Tm95cXJfSDFJWnBFd2gwbnVVcXg0SUMzVnRhRXZld3lTdHhYbU9lS1lwOXB4SGFZa1JHc3diTzZjZF82OUlwYlFSVzE5YjdjWW1PeGsxLTFtLTBiMEFycVFxa1hsalpwWnlGYVlkN0ltbnFUcVlqM3U2ak91M3FKWC1NZw?oc=5</t>
         </is>
       </c>
       <c r="F59" t="n">
         <v>1</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46055.38104166667</v>
+        <v>46056.22327546297</v>
       </c>
     </row>
     <row r="60">
@@ -2384,24 +2384,24 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AI deepfakes are reshaping cyber risk – and insurance must keep pace - Insurance Business</t>
+          <t>How trade shapes the winners and losers of AI boom - Oxford Economics</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:25:07 GMT</t>
+          <t>Mon, 02 Feb 2026 23:33:39 GMT</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNd0JwN0R2S2lhZk02UGFIVWlwODVoZ0NQZTMxZzFURWZURExNbmpXRFlfemNZTWpwNXFidktkSDlSek1EYzlmZzlRSGxoN1dxeG9vcmZYbS1PNU5qTld2RVNQZUNwMXlKcnROQUFXYmtmQUdoVUxxNmV2VlVDRnBSMEZtam1MUzFnd09sRG5IWkVlcW9JNXBzb25qUVo2WjVvRXdxdUt3VnZjbk5vN1hsNVpMTUNQMkUtOVR4QUc3M05NVUZKU2xzNmVn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxORDcwTnZjQkprcmdaR1dMYWE0TTlSZUJ5ZEVqOHJCZDhYT21QdG5veEJpa3lOWUE1QzRpaVN2TGQtcHR1dGtlV2xkc1lQSkFabUIweFhqVWIxWXNORVh2T1ZTVlJFbFlBbGNVRWdwZFQtMDh5MmIwUmdCUWU3cjFPZmRhTVhfZzBOZWlqcURqSTFQRm1XRHZV?oc=5</t>
         </is>
       </c>
       <c r="F60" t="n">
         <v>1</v>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46055.47577546296</v>
+        <v>46055.98170138889</v>
       </c>
     </row>
     <row r="61">
@@ -2417,24 +2417,24 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>One Identity names Gihan Munasinghe chief technology officer - IT Brief UK</t>
+          <t>Publicis deepens AI push, saying rivals have yet to make it pay - Financial Times</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:00:00 GMT</t>
+          <t>Tue, 03 Feb 2026 06:30:20 GMT</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOcnhlcVU0RWd5WDI4R0s5d0lvQmdaVHZQeW9QblFnTV8tYmJ2UjlWY1NCckNEWmZiR1lGc19GV3k3ZmMzaF9XV0IwQXBNSEp1N0hTQkhmcW1Wa2ozVmZGUDYzSHh4bFo4UzMwc2FzMmNLTXMzRWw2Y3ZkVHRxYWo4N214NThWRUhHRzN4eHRZbTB1UQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE05aFZudWF4Qno5cmZiX19mOXg2YWZvdlFIUVNjNHhsZGFfNWVxeEYzQmlxT0xud0hkYzdxSU1PRElxZHpOQ3o3Yng0aWYtS3FLdHhFcTJobU5oYTllaXI4eHNQS2ZncTNJeEJmd1loZ2Q?oc=5</t>
         </is>
       </c>
       <c r="F61" t="n">
         <v>1</v>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46055.5</v>
+        <v>46056.27106481481</v>
       </c>
     </row>
     <row r="62">
@@ -2450,24 +2450,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Breakthrough Power Module Aims to Ease Energy Strain from AI and Data Centers - Telecom Review Africa</t>
+          <t>Europe Today: European leaders in Dubai to discuss global trade and AI - Euronews.com</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 05:11:38 GMT</t>
+          <t>Tue, 03 Feb 2026 06:49:08 GMT</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi3gFBVV95cUxOQ293QzEtcl9tQWc2dlJOUG1MSWJwZm1pQXdxVnhiWHo4NEo3TU5YR1hzVXBGRXlQcFY4cDdfTjZPdXZBR3d1UDhXTkVtR1UybFotXzBPOUtDY3FkYndxbU9kODVOQ2RvcVYtM2FEeG80T2xLN1EwUVNZRTJkbzFBOXV5ZGRwRUJXcndkeUpfcDNLRnRxRWkxUHhiRjB6R0k2Zm9KRE1ENVh3TWZkcU5SYU1ja2NTZnJKOG52cndlYVdlN0REY2locnVVaHJLMnkwbXhERkROWTFFMzh3c3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxQeVpwc3ZyM2dISHFvMjNObW9wX2FCbDU1VXBNWGdkUTZXTW8yN0xQRlVGYldQaHNBRlNlSDVsa3dVS0V2c1Nkckdqa1RtQnBwWGRXVnRMVjBLVi0xcVlqemlJaVg1bW53VnhPay1kczBCVllFVW9vWXg3NDJub2M0bUJoQ1JzN0dRbUZaUGRaUDRBaHZxOXoteU9jc2s2Y0hkRnY2VGVkNThHVGFCVlB1akJwQmpxSE5DelY5MFpuQVA2WUxQOXc?oc=5</t>
         </is>
       </c>
       <c r="F62" t="n">
         <v>1</v>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46055.21641203704</v>
+        <v>46056.28412037037</v>
       </c>
     </row>
     <row r="63">
@@ -2483,24 +2483,24 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>EU Selects SUPREME Consortium to Develop The Union’s Superconducting Technology - The Quantum Insider</t>
+          <t>Large RIAs step up AI and data spending: Cerulli - Structured Retail Products</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:24:45 GMT</t>
+          <t>Mon, 02 Feb 2026 16:11:33 GMT</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxNaUNORlkxWXBCMW5YVjZIdHFFck9Yc2VhbGxWMElvaTI2RW01azg1cDBJTWlaclpXZENadEVsNXZiRnNpdUt3QjE5UkVkclByTTNEVXowa1VlTGZ0RlVIaWVIVkwzcjB6b1RVeTlkcjlWMXJrU2psMnNCbm1Fdkg0cW9faGpkVjFZNk1UVE1WejhXTjRfaHdaSUstY0k0UWZjeXNLYWJkbF9SUFRTWm9ZZTNXQ2VaQThROXlFXw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPcFBPNGFHby05c3dkYV9CNVZtRDc1eVdFRmhmSWdJVHQ1cE5GamVNaElKVnoxcHRSRFFFQnFyUDE2M3dzVW9MbmRCUmJVZnJsWXVLb1dMZ2xVa0VxUVNOaXJSNklRdW1oWE9RUEtabUt5MHJiQ2FrZHIxUGc1d21XOXAxeXJXZFFiLUtVeDJ1Uzl4VlJZV1VQczVJTzZ6d1dyUTdRX0xB?oc=5</t>
         </is>
       </c>
       <c r="F63" t="n">
         <v>1</v>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46055.3921875</v>
+        <v>46055.6746875</v>
       </c>
     </row>
     <row r="64">
@@ -2516,24 +2516,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Betting blind on AI and the scientific mind - The Transmitter</t>
+          <t>Barton Peveril case study - Google Cloud</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 05:00:58 GMT</t>
+          <t>Tue, 03 Feb 2026 05:13:05 GMT</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNdWJUT1lZS2tZZEVHXzlBbUJOaVl3Y2VLa3dXblRNcmxsci16YnBrWENIanhRRHFoY1k5VmkyenF6VzdXaGEtRW9WVFlwSXhtTFVHLTdLb1RGVTY0Y2dhZ3dWOHdPZDB1SWFNZnZoR0UyN05TNzQxYmx6eG9QRHROZERYX24tRVg0d0NKTm1OT1RRNU1WUTE0b21zT09UTW04?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE4xSjkwTjBsTk1qeWV5WGhJTFNIUEdKZkRXLUpGaFRUQXEzYVNNaUxkUEpDcmU1cFFJNjlCOVlkU2l4RTV1RmZsc19Sa0VaNXphVjJ3NFNMY1lmQThs?oc=5</t>
         </is>
       </c>
       <c r="F64" t="n">
         <v>1</v>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46055.20900462963</v>
+        <v>46056.21741898148</v>
       </c>
     </row>
     <row r="65">
@@ -2549,24 +2549,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>UPS Resets Network To Favour Automation And Higher Margin Deliveries - Yahoo Finance UK</t>
+          <t>The Telecoms.com Podcast: Ericsson, AI and Nokia - Telecoms</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 01:06:00 GMT</t>
+          <t>Mon, 02 Feb 2026 12:28:13 GMT</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxNaVo5eHdfOGZhUjJoM0RQeTBpbWNDb0NkdnZKclhQcWtCc2NJUGFmTVBZQmNwcFdibW9QY2JfVjVMTDRiMjNWRkxaU1VPd2hYOWlZSS1GUlJjWFlGMjBfVWZETUVBaUNsUENXVkJ4eDVBNVN6Y2dkNFRVSzBPQXc4dkFqZXNPR2d3QVV4SWRB?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxPTHhsYVpnTHdHNkNEQXR5YTVXeEdDSFh2dE9YLTJsdVdFbDV6MkxuQzJ5Q0xTdEZFb2VaMjlESi1JZDU1QWJpekR4ZExxY196ekhkZ2lJUDZzMnp5MjFrS250eDh5OGRSckRLczFKdjJKYVcyQlhmdEtSWTA2R0VLTTZUa1dhV2dlYXc?oc=5</t>
         </is>
       </c>
       <c r="F65" t="n">
         <v>1</v>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46055.04583333333</v>
+        <v>46055.5195949074</v>
       </c>
     </row>
     <row r="66">
@@ -2582,24 +2582,24 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Tarabut acquires Servable to add financial AI capabilities - Retail Banker International</t>
+          <t>Dow to replace 4,500 jobs with automation and AI as shares decline - Packaging Europe</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:43:07 GMT</t>
+          <t>Mon, 02 Feb 2026 11:08:32 GMT</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTE4zbkhCOEtya20wSGRvRG1UNHkwTGN0NmlmWFNXdUMzOThtTVdaUGhDeFh0T0YtdzlDa2dCdXFHYUkzdUJjb2d5dngySGY2aWl2Vko4Z0s1dUFJbHBUeFZVRGpOR1I3SHVMLTREeUJnS0VDR2NUTXpLbm9BdXBJZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxPUG85LWpVTTB1ajhzU3dMMEtCa3NkMDRxbmpjZTV4RmlvZ1dpSlh2VmZZSW40VEV2QzcwTDVaQVltdnpKT0gya19GT3I1VnJFUGNjRkNGNUtobGFCS0RjV2x1NmV5YTQ3bzlYUWxHRl81dnpLVk1vVHlEemtUU0JDeDk0SVhDYXBsSG9pMXBJdnJfOWpPQ3U4NjNVWm1IeEhCT1l6aWUxQ09EaGg0czl5MXh3?oc=5</t>
         </is>
       </c>
       <c r="F66" t="n">
         <v>1</v>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46055.48827546297</v>
+        <v>46055.46425925926</v>
       </c>
     </row>
     <row r="67">
@@ -2615,24 +2615,24 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Microsoft Q2 2026 Earnings: Can AI and Cloud Keep CX Ahead of the Curve? - CX Today</t>
+          <t>SpaceX absorbs xAI as Musk consolidates AI and aerospace ventures - Proactive Investors</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:46:47 GMT</t>
+          <t>Tue, 03 Feb 2026 07:19:00 GMT</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNUC1EZDJEcjROV0lVNzhneHVKWXk5NEcxZHk3OVZ5ellocGZJUnpTbHI2ZmNBbDVYY19SbS1XWGotdC1ISzE1S3RiT3dqWEFBY0JpUzlndDRCRlJ5SmdfZ2JhSlZQMUJsLUQ5UHA4NGZ3dlVKYmlRbnN6akZKSWZMbWxPWGtOOEVfZ24tMHBNMmZCam5ZeFhlRkkxd001SS1qanpXanNWM2xQQjNVaTRaV2Rvb0hLQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxOSktJdXEtMGNPWVJnb0ExNU9kLTNOVkhMei1sX0NVVjVuNXJYLWt3dVJaTXNwdzlaaERFemlOOTk1d1Y3d3oyQkJlQ2tEWHFFSnRIcDYzYVhIOE1JTkFXQ1J2b0NWRjRpVl81REJNUVlEeUhSb3VwYldETlFSUDBmdHRmd3R6N0FkWV9WVDV5TEw1YmkyWXhNNkNZREJVS09lVEhQRGM3SnBtdnVKbC12WHdselRoUnNtUV9BRkZXVmNBN0ctVjJWMGg1VmY2RWxaOWlVbw?oc=5</t>
         </is>
       </c>
       <c r="F67" t="n">
         <v>1</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46055.4491550926</v>
+        <v>46056.30486111111</v>
       </c>
     </row>
     <row r="68">
@@ -2648,24 +2648,24 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Why are women more sceptical of AI than men? New study sheds light - Euronews.com</t>
+          <t>SDAIA Launches National AI and Data Curriculum for All Saudi University Students - BABL AI</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:30:46 GMT</t>
+          <t>Tue, 03 Feb 2026 00:16:24 GMT</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPd285WTNKeFhFUUFjOW1qekVOX1dVeFBuZ1I4aGtZdjhsMFcwck00SGdRdHFkRmk5ZTM1Xzd1MDFtVkZYX29qRVR4RFY0Z21NTDhBRmhaZmV2azI5Uy1oTW9VbDRUS2thS0RYQWtLZDFIXzFiMGNNVjc3LXJNRk5CcTEzalNFQjNPUU1hbmRfcGJlRzZEd2I3c0FBMHFHVWltRDV3aHJBSnRZdWhPbVBfVmhKQVluQ1VCT1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOeTl0aUM3cjYtMFAzZ3IzU3VYRlJtWUVoX2ktMVJlLWxSMlpRcHVuWHdjNkdZNFh3cE56dXNvWjhXbEdNMGdTaE5PWHh1TFNwbjNCQzFWd044c1g0SmFFNHRzRWZwRmRuTG1FQUFtVUNHYWtISXdNWm03SlNDd1lWREtxel9RTHBicDQzVG9KMmZNUXBKVExBT0NCaHEydw?oc=5</t>
         </is>
       </c>
       <c r="F68" t="n">
         <v>1</v>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46055.35469907407</v>
+        <v>46056.01138888889</v>
       </c>
     </row>
     <row r="69">
@@ -2681,24 +2681,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CANSO Says Greater Airspace Capacity Requires Automation and Strategy - Aviation Week Network</t>
+          <t>IFR position paper on AI in robotics released - International Federation of Robotics</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:39:01 GMT</t>
+          <t>Mon, 02 Feb 2026 09:50:47 GMT</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQeEpFajRYUjU3cDhISm9odXVmaF9BU01aZFZxNndTd3AyUnJyZWV1MVdsbjQ5SEt4UlZ4LTJTTFkxdW9lR0xITzY2TFpWQmJiRDhYTzNyQnJhWDNhY3g3bTQwdHVXd3J5ekFtdnlJZ3M4ODU0NWE0VFllMHRBTEpUbTh5OWJBT3cwcllYWHdlZ00yUFNOX3lSNGtKZk40aXpBVzNSVllCeUFmeDkwaVdSM1pFMTZsbEp5SFkwOFpfbw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE1uM2Vnek8zdm5IV1hWem9CYWl1S0czMEJLd3lhNHNlLURxajlQZy1ISzdSd28yblRfeUpKV3ZsYWlPYlJsNGdDalFWMUQyOTVqSmQxMzNqV1Y2SE9UbzRxcjc3RzVRcTc0NG9tYV9JbU5fWVAzemRVMTVhV1o?oc=5</t>
         </is>
       </c>
       <c r="F69" t="n">
         <v>1</v>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46055.5270949074</v>
+        <v>46055.4102662037</v>
       </c>
     </row>
     <row r="70">
@@ -2714,24 +2714,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Maxio Report suggests B2B SaaS and AI growth remains strong but has become more selective - Enterprise Times</t>
+          <t>AI in 2026: From Promise to Pressure - Teneo</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 07:14:23 GMT</t>
+          <t>Mon, 02 Feb 2026 20:55:49 GMT</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxQS1Y4c09NU1JsSUlBMjFudjlEUGlkX19mdWR6Wm5pZ3VpV0NMd0JFTjY4YmtPd1VqWjRzb2E3aGNyMjlxSlBUVm5aMnl5Z1RabC1rNEZpcW1mSURYaUZVVko5dUNkQ2kzekltTDR4dHpTQS1uZFFHN2hWYS0zYnl1NEp5UERRczJwU2pKUnkzakN3c3RZaXM2R3EwX0tXZWgxcUlVRmRwOTc4OGxacmRWbjM3WXNQaUNYcnhwOXptTXpHU2RpRWpNaVEwUEU1UzZR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOLXVwemdRYk1qT1FqeUh0VnVrQ3dZWVNmWU1jWDJFaHVRRWlUcW5ZbGowSXN4MFBaSGwyb3lkMEF5aHg4VXdpRWtrNng4b0dIWldJdUJBRl9MNkNoRndQMGQxVVpub1p1VmRUekJodHYxNnpZV1M5NFV5REJiaU5fMERPQnlkTEZ4NUVKcFA1QUxXYTA?oc=5</t>
         </is>
       </c>
       <c r="F70" t="n">
         <v>1</v>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46055.30165509259</v>
+        <v>46055.8720949074</v>
       </c>
     </row>
     <row r="71">
@@ -2747,24 +2747,24 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Grok, AI and “free speech” – Starmer vs Musk - palatinate.org.uk</t>
+          <t>UK-Bulgaria: connecting semiconductor expertise for growth - GOV.UK</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 20:30:01 GMT</t>
+          <t>Mon, 02 Feb 2026 13:59:31 GMT</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiekFVX3lxTE9Qa2J6bG5BUjIzZ2k0Zkl6Ynk4a0x3dl9Hbm1yenJMNE1iUFM1cVY4d0hUcmdwYk5XRTB5a3ZjN0h6eldTVU41TkdWV185ZzFLQ0VCZkdkVU9keFZubF9kV0ZsQUdteE5jdDlKdHRpdUdjNXRacVpwMDR3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPUHdYRDVQYWVLZjR4MnFna1dPMEJYd25Bc3VvdllKVGJ3OXAzcGIzUy1zX3hQUHhfZVdlZExSZWVkVUc1dGF0OG5ncVRpNkp3YlNaaFBKZjczUm1ET3hBMVlRR00xbi1oVTZtS3REQ2tjek42Y1lKQUdTclFzT2dobGhIdE55QjVsVzFqTUJ3U01aZGVISTU0?oc=5</t>
         </is>
       </c>
       <c r="F71" t="n">
         <v>1</v>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46054.85417824074</v>
+        <v>46055.58299768518</v>
       </c>
     </row>
     <row r="72">
@@ -2780,24 +2780,24 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Can agtech fulfill its promise? World Agri-Tech explores opportunities, challenges for the future - AgTechNavigator.com</t>
+          <t>MediaTek Accelerates AI Development With an AI Factory - NVIDIA</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:06:00 GMT</t>
+          <t>Tue, 03 Feb 2026 06:16:43 GMT</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisgFBVV95cUxNWFFRQ2RucW80azhrWVJ4Y2J2enBFdDJHOTVlcXhnNWtDTmJsOWdadnQ0cUVHNzRXSGhlUGZweUI4RlZGWHA2cFRRRUl6YVhxNzNFYVd1d3dMMFU0LVJXbTA5Zk80ME14ZGhoVjdpVzRXUFZtV0pWb010Z2kwZWliVXV6Z0FkYlBqSmN1b3F6YklmTWxVWWtpVzh0RnhCYWZ3Qm9KLTlrUEFJUnBtdkNrVVpR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE1EY3BvY0lNOWlaSGhoYWRHOFl2ZVBVZ281bDRzMXJtT0FTUzhxYkRmMU1WaEJkWnpGN0kzYzdPZjBqeV9qQ3hQdXpEUUlNRU51a0llSWRpLURiLXVxbHpfTWxKNUpxWV8yYS1tNkdHSQ?oc=5</t>
         </is>
       </c>
       <c r="F72" t="n">
         <v>1</v>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46055.42083333333</v>
+        <v>46056.2616087963</v>
       </c>
     </row>
     <row r="73">
@@ -2813,24 +2813,24 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Tesla Recasts Identity As Robotics And AI Platform With Merger Potential - Yahoo Finance UK</t>
+          <t>The Balance Between Rules and Learning in Robotics - Telecoms</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 17:10:27 GMT</t>
+          <t>Mon, 02 Feb 2026 16:52:45 GMT</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOenZGbUM3RXE4U3Q5RUU5bmZoOC1MelduTGw2Nkl5dWpLZVY1UmNPWnpxQU9Pam1IWGtaYndOcUZWSGt3amdtZk1MQ2hOXzQxeFRETlRFWDd3UkxienlDSWhhTHN2c0hSblNnckdBaUg4V0JOQnlYdjU1VjliMF9aZ3gzNXpvQ3p0RVFR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQVGNhZGZTZzZjUkl0NlJQWmpWSmFOTGlRTm9DZ1VDbXl1ZUs1TVBIT2ItbHdyV19ULUJDMWZfTkFGS0tuYWFyMGxTMEtFTEhFSXNYeUxYNGdvcmYxcGZ3ajdJYzVYcTVDQ3RlQTlwOHVkekljNUtOYWloN0hEZ2lfMmgtRm0?oc=5</t>
         </is>
       </c>
       <c r="F73" t="n">
         <v>1</v>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46054.71559027778</v>
+        <v>46055.70329861111</v>
       </c>
     </row>
     <row r="74">
@@ -2846,24 +2846,24 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Managing the Load: AI and Cognitive Load in Education - Faculty Focus</t>
+          <t>30,000 at Web Summit Qatar for AI, quantum and creator economy - Euronews.com</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 04:07:18 GMT</t>
+          <t>Mon, 02 Feb 2026 14:58:41 GMT</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxNNUhwYkZCLS1OQk5FMnVLNThFcE05TGx2M1lEbld3bEdyT3dYdER5b0dwMnJZZW83YlBGRDIxYTRWRXp5eTJHRlRnZ0JwS0FzTHFRV3ZQRV9ZNGVqendFYmN0ekE2REVEblRMX0xWTGlUXzVsWGJLYXFjSkcyaEh4ZGt4SHZXQUU5bUFsWDgtelExVEV5bklDaHZTNk43RDkzNWNTcWwtOGZNYWlLTnY2SXhXNmtPNk9tMVpqWG1n?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxPUEx0MTRuaVlMOHV3YkdXb182cC1BZE5OMVFMekFxWVQzX1l4UkpJTFBtWFdVYnU5UDVnUTlTelR6ZzFnd3prVVR0cXlScThjV2Z0TGswU3RoeXA2TUhfdjB3alhVRllMTDBIa3d3ZjhISGxrbWNJVjl5M29YbTFjTmpFSndVWHRPZEpJVWhTN0VGWWM0WnlCX3hNcHV0QXB1QWpqaGE5dWsybWFGV3dOMw?oc=5</t>
         </is>
       </c>
       <c r="F74" t="n">
         <v>1</v>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46055.17173611111</v>
+        <v>46055.62408564815</v>
       </c>
     </row>
     <row r="75">
@@ -2879,24 +2879,24 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>C-suite poses greatest AI risk to businesses, not entry-level - Personnel Today</t>
+          <t>Electronic Design Automation Software Market Size to Lead USD 34.71 Billion by 2035 Driven by AI, Cloud, and Advanced Chip Design - Yahoo Finance UK</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 05:00:58 GMT</t>
+          <t>Mon, 02 Feb 2026 15:02:00 GMT</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBhS2t1cTV0UkhxRmkxdkM0ZmU3eU1JUVR3WG5wY1lkMm1lNGZUZm85VDVYUEFJQnZmVGhKY0dfQkhGWjQ3bDk2bWdZSXRHM3U5ekc4LV9NNGs5MUc1R2owQWwtRlRUSlYwSXluN2VBTVZpS3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxQNUtvZDlhS1BqSDdfeFVBY1ZaVFNMd2ZOX3QyQk02UGtkNDFidHNkV3dLRXlVdEI4R0JjYkI5MzZiR242TVg1bTRJam4wakR6UUdJbzNXZmYzYUZhcC1JOV9EaTM5dWh4Smp0czlIaWJKYjRMNkNJQVlyMzN1V3QxUy1HbEhxRmF3QzUzMW8zaFJHSzB4Z0RJVw?oc=5</t>
         </is>
       </c>
       <c r="F75" t="n">
         <v>1</v>
       </c>
       <c r="G75" s="1" t="n">
-        <v>46055.20900462963</v>
+        <v>46055.62638888889</v>
       </c>
     </row>
     <row r="76">
@@ -2912,24 +2912,24 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>AI’s ongoing evolution in corporate travel - PhocusWire</t>
+          <t>The power of putting AI governance into practice - Global Government Forum</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 06:04:25 GMT</t>
+          <t>Mon, 02 Feb 2026 17:11:25 GMT</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQNnRpVmpSMDE0TWZYaXlNalhkMHN6VzdTWGJtbGtXdnd4bUhzZWpQS3dDUFVZaDdteGJxNGUySnBwMkJuemQ0U1ZVVF9XX2U2bktCa3BxcFdKQjBIOVZiUlhldm52YWNBOWpneWpQQWZXMlZvOFRiYXVJTTAxVndtdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQWGllM2ZaRVR4MDZreC01cWFWUTNoTW5fMWc3bGVxTVVkSjVzNXR2cmp1UTlWM2ZDQjZHckNkVTIxdTVnQXZXc1JsTWhXSW0xWDB2dEtFWUNNNjE4emNveHN2dk1hMHR3VlJVWkVzSXRHMmd5Z0d3NUhQTFpGQlJTVGNFZXZvaDZnTkU4R3RqbmI?oc=5</t>
         </is>
       </c>
       <c r="F76" t="n">
         <v>1</v>
       </c>
       <c r="G76" s="1" t="n">
-        <v>46055.25306712963</v>
+        <v>46055.71626157407</v>
       </c>
     </row>
     <row r="77">
@@ -2945,24 +2945,24 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Deezer opens AI detection tool to rivals - Digital Watch Observatory</t>
+          <t>Christian Klein Bets SAP’s Future on AI and Data with 5-Point Growth Plan - Cloud Wars</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:05:00 GMT</t>
+          <t>Mon, 02 Feb 2026 16:00:00 GMT</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE9ackFocUVZY1ltM2ZxaVpSQWFCcmdGTGVmRkN4WW10LXZJZlVFckQzQnc5RElZWmNvbzhPTEZVbFFLOGdwNm5RcE5ncmt3UkxoUXRRVzluTnlRMndvcXNYNmVQY01XOFpZeVlzck4tSF9TZTIy?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQU3d6S1RPNFdFbzJkR0Jfd25KTmZ4dW9lQkozcVlCS0ZPa2xOc05WWmhTMGJYbHlFVy12d2hnb2h2cU1XSmlrWC0tNkpHSEtpcENPRElUYlkyWXE5ZXd3Z2M3OGVXd3FRUDdWaldfNGtfc2FsMk94WmNqdnRONnVEY1k2dEpTeWViTmxyUjdYN1ItcEhuMHVZN2Y2OW53eUJrWXZGcEJ0cS1sSzNXS29qZnlXNnlmVHZO?oc=5</t>
         </is>
       </c>
       <c r="F77" t="n">
         <v>1</v>
       </c>
       <c r="G77" s="1" t="n">
-        <v>46055.33680555555</v>
+        <v>46055.66666666666</v>
       </c>
     </row>
     <row r="78">
@@ -2978,24 +2978,24 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Kazakhstan to Introduce AI in Water Sector by May, PM Bektenov Says - The Astana Times</t>
+          <t>Forfusion Partners with Stellium Data Centres to Accelerate AI-Driven Innovation in the North East Growth Zone - TECHNOLOGY RESELLER</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 12:37:49 GMT</t>
+          <t>Mon, 02 Feb 2026 21:07:25 GMT</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNT2JBTHhOTmhnTTBtcWQ5NTVCR05aeW5oZnlxNTlyQzVYbllIWHdXX010Y3R5amFnUEN6U3d6Q1R4NVZZMnVhUVJiM3pmWVUyRzl3UTh4WUhwQjV4LUlRZ0k2TmlzUWx5QkhWdl9UbTNvUmRwNUM2VE91a3dCZEpmQlBqMVdSSlNpdnF1RHZKcTZ2UjRBcmRiWjR2ZWV2TFdu?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxQc3VIdlFiZkpoWTlVLW41UW5aaU9Jb0ZzZTFCOURUSm9maU9Sd3hyWmpkZVROdFB5RFF3UjJEUHVia1FWdFNzdUhYczFFeUlGeXk1Zkw4WE5DSkp2dkNEc1ZOT2ZlWjFXZHlVMFhSMzRubVFjempHQmU1M2tuaWZvUEhmUjBKSVBpT0FfalRta0JfQnR2MDlJdUlhUWtrMnZ3bElJM2hnUlotZDdFd0xOZEdDX0FiMUNhMFplM0pmQ2ZObENSQkRqclAwSkE3SHpVcm4yUU43WEY?oc=5</t>
         </is>
       </c>
       <c r="F78" t="n">
         <v>1</v>
       </c>
       <c r="G78" s="1" t="n">
-        <v>46055.52626157407</v>
+        <v>46055.88015046297</v>
       </c>
     </row>
     <row r="79">
@@ -3011,24 +3011,24 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>China, AI and the West’s Free Speech Crackdown | Ash Sarkar Meets Ai Weiwei - Novara Media</t>
+          <t>NEWS: NHS Tests AI and Robotics to Speed Up Lung Cancer Diagnosis - Practice Business</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Sun, 01 Feb 2026 15:03:30 GMT</t>
+          <t>Mon, 02 Feb 2026 08:38:49 GMT</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxQVlRxZHhhcHV0NGFidnJRcWZkQnc3WWZLQkNiR1M0T0JSZU9MaGc3VkprNWVvWkZfUVpaaHFxUVFHdkpjdUNWSWRiYno0cXhpOXZNWWF5LWJCV3NzRVJCM1lhbkc1YkFmNUg4ZG9FZ3p4RTJEZUNKeUtIVkh1cDVzTzdMQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNV2k0ell3bnhNOFBMM29oU3ZHenZTNkFvX0lDc01hSjN0QmZFM053cndMN3pPNDlPOGRxNUVVMjBuSDEtc3hSSXRzNkhwdkdMWlFvUzBGc08yWVM3S2tvaW9fd09heU83T3ZKVzF2NGpPc3VRamZzbUVMZXdqbUJtMm8tcDI1d1ZrM2RXTDU2VUZ4OUFMV0hkbEY4WQ?oc=5</t>
         </is>
       </c>
       <c r="F79" t="n">
         <v>1</v>
       </c>
       <c r="G79" s="1" t="n">
-        <v>46054.62743055556</v>
+        <v>46055.36028935185</v>
       </c>
     </row>
     <row r="80">
@@ -3044,24 +3044,24 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>KPMG warns of gaps between AI ambition and returns - Digital Watch Observatory</t>
+          <t>Energy, healthcare and utilities: how to tap into AI in the real economy - MoneyWeek</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:00:00 GMT</t>
+          <t>Mon, 02 Feb 2026 15:58:55 GMT</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxPa0NUQkc4cm94QjhSZ1ppc1Bmb19FUW9RTGNjWDdGUHJncnFpeXNFdkJYS09LTHk2dGRQVUkzb2ZyMGxYOVJyeXlXSzJyMGwyTkdQOVpjX2NDVHMwalNMTkpoWTdPbm1NR1dRRDNKQ1pGbnBBZ1pzOVlRalJCM3dDQ1p3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE1xc2lydjV1aDZXaXliWnM3UHJDcncwYVF4Sm5QMWNxM2ZHb1J4OXNYYzJhSnZ1a2wzSDlBQ2UwWFpGWUlESkRQeV9PME1TUDRlOVhLZTVOSjdpU0Z0UUlWMXBYS05UZDZ1UmVtN2NqTlFwaXV5bEE?oc=5</t>
         </is>
       </c>
       <c r="F80" t="n">
         <v>1</v>
       </c>
       <c r="G80" s="1" t="n">
-        <v>46055.375</v>
+        <v>46055.66591435186</v>
       </c>
     </row>
     <row r="81">
@@ -3077,24 +3077,24 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Venture Investment in AI Rises Fivefold in Two Years, Says Latest Report - The Astana Times</t>
+          <t>Answers to key questions about AI in IT security - Computer Weekly</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 04:52:40 GMT</t>
+          <t>Mon, 02 Feb 2026 16:59:23 GMT</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxPVHdSRUZ1LTFkVDJ0VE9td2pIY0xHaThneU82YXFyN2Ric2JQSWpjTHY4WjR5ZDlDbXVMZHpVbTRvLWlTQnl3WlZYYTltYjh2ZGJuYTRkbkNoa0N6ZFV2MEU2RVNNZ0x6b3NoU1ZvdGRiX3QyVmpPNG0wREpJVEZ3VmZ1QS1VRWI3NWN6UXg1em96UTVkdjJVUTZSOXl1ZFF2MHE0ZTFwVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxQenRxTzlpYTV3NW5xVEVqcFpNRDhZT1ZQbUFVdjQ1WFA3Y09MenRmUUd1MTJlX2NSTy11VUN5YzhmQkNyUnZCMG5kQTFYYTJ5aUtjcjlQLVJmQVZxbDUtSzliY1lLaVFfTzlzSTVLSHpKYk5DbzdzMG5DaUU3X0VYWklOemd6NmZ5M0JpaEF2SFk?oc=5</t>
         </is>
       </c>
       <c r="F81" t="n">
         <v>1</v>
       </c>
       <c r="G81" s="1" t="n">
-        <v>46055.20324074074</v>
+        <v>46055.70790509259</v>
       </c>
     </row>
     <row r="82">
@@ -3110,24 +3110,24 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Who Answers When We Ask AI About God? - EWTN Vatican</t>
+          <t>Why banks shouldn’t wait for AI to fix the Gen problem - Retail Banker International</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:26:40 GMT</t>
+          <t>Mon, 02 Feb 2026 09:28:04 GMT</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFB5NklNUjczbU81ZU1UdzdnaGdKak80OFJseVEyX2hKbUY2VVN4VUJBSGtBcUo2NGtTYkIxMDVsUHE0TlRfNlI1ekRScDExMjNDbHdUeVpVbkI4TTBPV3Z2NHpoakN5OVB0LWgzVlBlS0txeGJIN2RqemZfVmlkdDg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxPNkJaSEM4djg2STlSalNWM0c3MmhmS1ZNS1c5MG14VUREZzNha25fVXp3VXF0YUczMkRlMEwtVldORHU4TFA1dEtLY3dfeXpmcW5UbHJLR09mX3FYZlFwbmtCbU1GZ3lsMFBUZmhpU2ZHMzlVZUxkSG0wNkRCeFcwQkk1OW5ZUlVaNXFPVktQb1g0djI5ZkQzU0ZKTQ?oc=5</t>
         </is>
       </c>
       <c r="F82" t="n">
         <v>1</v>
       </c>
       <c r="G82" s="1" t="n">
-        <v>46055.35185185185</v>
+        <v>46055.39449074074</v>
       </c>
     </row>
     <row r="83">
@@ -3143,24 +3143,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Opinion | Where Is A.I. Taking Us? Eight Leading Thinkers Share Their Visions. - The New York Times</t>
+          <t>Year in Review: 2025 Artificial Intelligence-Privacy Litigation Trends - WilmerHale</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:03:00 GMT</t>
+          <t>Mon, 02 Feb 2026 18:05:23 GMT</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxPXy1tbFc5V2p0NVlhcHJUc2FQeFZkS21UMjQ5NXdkcUZib2VndHZOenBpTW5uOGZvYTRoUUZSN2tZT1c3M19XbDEtbkpVY1pPbWJmdmp5RDZuVFZtWDkyb0ZhbExleXl1NnBCVTJWSktzRHhicldUMnFOSmpLOXdLck5waWpnTUktenh4WmRsZExTdkNELXFwVQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi9wFBVV95cUxNelJqZWo1aVZoN2ZxMjJvckNuZW85ZzJzWTNhaFowc2swaTZLc3dzRWJ2Si1Ya3NXSDBfeXJLOG1NVjVVV1FHV21TZXB4clFKX3ZUTnEwbTIyN1pDblVSQnRSYTdUdmNvQmZWR21BRDdfQmVJd1J1VEQ4a3VmVVZlQm40XzZQZXlEVEJuZ25QemoyVnJlVWtBUkVUSTVJUEQ1RXpYN3VHZHhmTmtCZlIydmhZRzBWM1RwOE9nWGZRanc0WjNUaXdBdWg0UjJXUUZNbW1wcXFJOXNHbVVCUE1YLVNZTGItd0VwR3hLeExudzlpNThYaHJN?oc=5</t>
         </is>
       </c>
       <c r="F83" t="n">
         <v>1</v>
       </c>
       <c r="G83" s="1" t="n">
-        <v>46055.41875</v>
+        <v>46055.75373842593</v>
       </c>
     </row>
     <row r="84">
@@ -3176,24 +3176,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>How AI is Revolutionizing Life-Saving Drug Discovery - Pharmaceutical Executive</t>
+          <t>How sustainable funds are navigating AI, defence and financials - Trustnet</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 11:06:40 GMT</t>
+          <t>Mon, 02 Feb 2026 11:01:33 GMT</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOZlkyRDlhc3RUM0EteE5ObTBkSE9IUmZGMzBjX3VYYmZ3bW9oN0x5aWRFYWZfMTdpRmNMZGxYYmNLZjhLZEZLNlNRck8tdXR3X3Y5T3BDV0hubWwwMlE4NFV2Tm9OM0wtcUowUDdpcG5aUVF0TW53QkQ5M1BZLUJVVjJrbEo?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPRktGQTJJdXpHeldsX3E3NEl3ckx2QjkxU2tIb3lPUF84dEI0a2ZfQjVjbTNMeHpZUFZjdkR2bldWTnpMRmNjMnBkNFZ5Rk05dW5xeEpsTWo1YkRXUjhpYkdEYS1od0dPSmhScjZPRjZsYVBxTzlUbXh1QlVrbVhwaFRyNTB4aEk4V2I3b1dhV1J4VC1vRUdsMmdTUEFFeElqbE1J?oc=5</t>
         </is>
       </c>
       <c r="F84" t="n">
         <v>1</v>
       </c>
       <c r="G84" s="1" t="n">
-        <v>46055.46296296296</v>
+        <v>46055.45940972222</v>
       </c>
     </row>
     <row r="85">
@@ -3209,24 +3209,24 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Starbucks bets on robots to brew a turnaround and win customers - BBC</t>
+          <t>Yaspa Becomes Founding Member of UNLV’s AI Research Hub to Advance Responsible AI Adoption in the Gambling Industry - FF News | Fintech Finance</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 00:11:06 GMT</t>
+          <t>Mon, 02 Feb 2026 15:09:39 GMT</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5nSFI2ZTA2QTdDc3FqelRieW9rT0N4OXU1Mmc3YmtLd2V0Si04SmtQdlVqOG50ZEJKR1NnXzA5YmVjQUk0elRaeXZuZi15cl9zYTV0VUFRc1pMQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxQX0k2RTd2eVNGVVlxZTEzYnJKZUR4QmJtMjdTVHNmb2tha0pVbVFpOVduV2dWWFVha183MGRuRjRnc1NCVGZvcGcxYnBRUnZrd2RrVlAtMmpjbnU3MzFIYW5NUUxqbnJSQkdab2M4akJVMERVQVliRGZGZmtvT0FhTFVwZlVLMWlhTDFDRDI5bzNPbzh0cjlfemh4Y1pvZC13ZGI5cU9OMEhUT1kzZmd6QVktRWN2QVpUd2Zla295cm5TZzR4Uk5SMENPSU9PRG81MjdNd3podUxlVmUteWdRTjhKaXNibmNmeFE?oc=5</t>
         </is>
       </c>
       <c r="F85" t="n">
         <v>1</v>
       </c>
       <c r="G85" s="1" t="n">
-        <v>46055.00770833333</v>
+        <v>46055.63170138889</v>
       </c>
     </row>
     <row r="86">
@@ -3242,24 +3242,24 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Is AI killing productivity? - InfoWorld</t>
+          <t>From Ideathon to Pilots - Updates on AI and XR Medical Education Projects - Yale School of Medicine</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 09:04:02 GMT</t>
+          <t>Mon, 02 Feb 2026 13:35:17 GMT</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifkFVX3lxTFB1VTZOQWpQSWhQbjRZQWZyS0pCbkxuWi1EVHhQSWtKV0RmSTAyeENSVGVrcklaZnJLTUxuaGVBSHJwTnYtWXU5VVlFcGJPVC1qdWQzNzRsUXJram1GdHJCQzVHalV0ZFhZd1ptaWhabUtrd1RoRlNVUFoxZ1V2dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxQLUdWWXRPYW84MkNFNmV2c2s1RllLSXh1azlkbWhHVjdpM1RkbzBHUTdINWNQckdDVWNEdmxGaVZhczRHLVh1SEVMNWgtV3NNOEIzaXh4WENHNEN3djRwbU5ZVDF5VkpwY1VrOUI1dVJHaENlQmlqVjh1SXVQNmpXWklBZjROZ0tpVU84b25R?oc=5</t>
         </is>
       </c>
       <c r="F86" t="n">
         <v>1</v>
       </c>
       <c r="G86" s="1" t="n">
-        <v>46055.37780092593</v>
+        <v>46055.56616898148</v>
       </c>
     </row>
     <row r="87">
@@ -3275,24 +3275,24 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>How technology can help bank Africa’s informal economy - The World Economic Forum</t>
+          <t>Policy in a Strange Land - felixonline.co.uk</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:00:00 GMT</t>
+          <t>Mon, 02 Feb 2026 19:27:01 GMT</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxQY2VyZW5aLWxNNlhIajNPWXJfN0ZCSXh2T0xWSTdpX01yeUxoMGYxVl9tQ0xZdXhZMWJnX3JYMHg3YUkwZXdDdHJRTlNGLWtDM2doendjWTJKZVNmZjFxejlSbEYtalVKX0o0MVVUYjJIZVhNMkZFelIxem5DXzhzemZ2b0QtcHY2ckxrZG0zQ3ZLSnAzbkozOXhkZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE9KSXF2Z0M1YUtkQUJLOGN1RTU1MmVrbkc3cFpSS3BiU3RzTXhWUW9FZjNEYTJJVUx0elRZaHhfdGhNN09YOHJLN1Ytc2VEeGwwU1FKSnczRXp2dkVTZ0JpVGVwaFlNb05lOFZodQ?oc=5</t>
         </is>
       </c>
       <c r="F87" t="n">
         <v>1</v>
       </c>
       <c r="G87" s="1" t="n">
-        <v>46055.33333333334</v>
+        <v>46055.81042824074</v>
       </c>
     </row>
     <row r="88">
@@ -3308,24 +3308,24 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Did artificial intelligence really drive layoffs at Amazon and other firms? It can be hard to tell - ABC News</t>
+          <t>What is the 'social media network for AI' Moltbook? - BBC</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 08:27:13 GMT</t>
+          <t>Mon, 02 Feb 2026 13:59:14 GMT</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirgFBVV95cUxOUnd4UzhaZlNjTEVyRDVIbVgtMFJJcExLR1psMVdtWUxYcktJX05BUkFISUJLdW11Z09DYkg4UHhNVXdPc1NzdVI4VTdDWTBVNE5qSFVWRmU2YUtSSDFSWTJRM0pZWTd6YVRnQTRfcF9lUTE0VHVqX0N4TjFYS0FTSGdfQmxkU0IyekVEdnJjaXlLb2FaMHpLb3pKclJFbkktX3MtTmtlRDdzRWVHYlHSAbMBQVVfeXFMT0lRTjhydFNjTllyUF9qalVtbW8zSVdvSUpJcS1fMlY0a3dFb2VhZWtzZXhXMzdXeXVYUHd5TzNBTDRWcmRHM0l2d21yVkdhZEVLWFA0cGJHWG5hYkNTOHpMNFRhZkpIcktLVnUwUExqSlN0X1BkOHQ4dk1oWGdFS01kOXlKVWxYWGdVMkRnNHlVV2IzWUJVVDE3LXRDWXF3NWViTm9OOXlWOGV6aFVEb0pHOWM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFB3OWtDak5HWnlsTlhORjhSSEp3cGdyUzJaUU05cmdlTlZSTUZYclByUUFaWDh6OGdoMXRkYk9KRmFmbEp6SEpYd29uaEtWY25HQktwdFVTbzhMZw?oc=5</t>
         </is>
       </c>
       <c r="F88" t="n">
         <v>1</v>
       </c>
       <c r="G88" s="1" t="n">
-        <v>46055.35223379629</v>
+        <v>46055.58280092593</v>
       </c>
     </row>
     <row r="89">
@@ -3341,24 +3341,24 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SPIE Photonics West 2026: AI Everywhere | Business | Jan 2026 - Photonics Spectra</t>
+          <t>“A cloud-enabled, digitally resilient Europe transforms the protection of its citizens, infrastructure and strategic interests” - Thales Group</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:28:00 GMT</t>
+          <t>Mon, 02 Feb 2026 12:00:00 GMT</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxOVER5ekZJMjhVaG1QdWFaMlNMU3R5QjY0U2RkY1JqQllOVDhOcUJQaHJOOEswMks5dmdRWHB0ZlNjV1dRa3BxRlZ0SVgyeXYxaTBQQmRpWEx1M1NfZlh2bmoxaUF3YzkyZnJXWlhDX2o0QlZ0bGdHY0NhNnlvRUZrWFJDR0hkaU5aRnBN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxQc3lvdXNHRWx4aTVFNFlPbGUyTjB5UlVaN3dhSUhvbXQ5dmF1Tk91REd1QTU4R2VPbGc0b0VEbTZrRlE0cHJWaXVFYmlXaDFDMDhqM3BUOWtNZzJLb0FBSEh3T2pwLWEyTE5ycEpEX19mSmJ4TG40UTIzRVdZTk1IdEpFaWpfVmtoZFRTaXRBREk1YzdNdk1NOVJFRHpzdTJPemlFYmZiWGtuWEJJWVgyaVlDSDBsRjFoaVVUU2tjLU9ZUQ?oc=5</t>
         </is>
       </c>
       <c r="F89" t="n">
         <v>1</v>
       </c>
       <c r="G89" s="1" t="n">
-        <v>46055.43611111111</v>
+        <v>46055.5</v>
       </c>
     </row>
     <row r="90">
@@ -3374,57 +3374,288 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>How AI Is Changing the Storied McKinsey Interview - Business Insider</t>
+          <t>Confronting AI: The Future of AI Regulation and Your Path to a Career in the AI and Tech Legal Fields. - UC Law San Francisco</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Mon, 02 Feb 2026 10:31:00 GMT</t>
+          <t>Mon, 02 Feb 2026 17:23:12 GMT</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxPTGQyZlRzS3c2MDdEQ1JKaWIzYlFkOHZEY1JKZWx2bkRfRTBLQW9mTGM5ZWk2dmFXQnpVcHA2dEJ3QTBQRkVRQnVJMjhSejFKdTBXbHh3VGlRSGMtcEh1S0hhNnktem5VLWZFTEJGdUI5SXpDUTBHdEF3a0NoUVhSMXJyMk5ac1U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxNbm01cEhkZjg5ajd6M1lsYUZFbEFHMkRDZEwzYVQ2N2xoalN6S1FZSm9QZU1CS3YyUGg3cVZuTEt3UWVQYVFkeXN2Y2U2bGI1R0pqVExjRGdqTFJGcm9GdFpQdkdCN1dWZDQtaG9hQzhrLVJ4TFFBNlNPYndWRWlGRUh5WXAxeDFzdU5WYmJlTnZPWGlDeUZ3ZjJWSVV1TWdIOE9Rbkx2amFjekpzY2FhZTA4dXVzc2xZSnZFakFwd0JEanRvbngyMldnYw?oc=5</t>
         </is>
       </c>
       <c r="F90" t="n">
         <v>1</v>
       </c>
       <c r="G90" s="1" t="n">
-        <v>46055.43819444445</v>
+        <v>46055.72444444444</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>From Performance to Purpose: Lombard Odier on Intergenerational Wealth, Intelligent Technology and Enduring Partnerships in Asia - Hubbis</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 16:04:12 GMT</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi7gFBVV95cUxQS2puWGNpajlmcGtCMnhvcUo4MHBxRWJiMXlBRjFjLW5XZkRUY1o1MkkyV25mV0Z0bkYwcDY0anFmR29qa0NnWDAxZVc3MkczZTgySG1rQWx0OFVEbWtxd1d4UlRfTk1fZDdGRHJVQkowcVZsZTNLUDN4YlFYcE5RSnhEMDhvT3hqby1ESXJ6R0ZXS1ZxMklPVU9aYXFpeDVUTzBWcUFCTEtDYUJVWDhCYnJNVHhrdDY1RUxFa3ZDTFUzUUpnMFV2OFdqSzVFaWU0aTZNM0VKZTJ5dF9ZUXhHanVESzFFdTdqX2Vyd2ln?oc=5</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="1" t="n">
+        <v>46055.66958333334</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>AI deepfakes are reshaping cyber risk – and insurance must keep pace - Insurance Business</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 11:25:07 GMT</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxNd0JwN0R2S2lhZk02UGFIVWlwODVoZ0NQZTMxZzFURWZURExNbmpXRFlfemNZTWpwNXFidktkSDlSek1EYzlmZzlRSGxoN1dxeG9vcmZYbS1PNU5qTld2RVNQZUNwMXlKcnROQUFXYmtmQUdoVUxxNmV2VlVDRnBSMEZtam1MUzFnd09sRG5IWkVlcW9JNXBzb25qUVo2WjVvRXdxdUt3VnZjbk5vN1hsNVpMTUNQMkUtOVR4QUc3M05NVUZKU2xzNmVn?oc=5</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" s="1" t="n">
+        <v>46055.47577546296</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Whether it’s Valentine’s Day notes or emails to loved ones, using AI to write leaves people feeling crummy about themselves - The Conversation</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 19:05:03 GMT</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxObU1UcmpiWm5TdXBWNGtVV2JaODBFWUZhamtxaHFYU1M5YlhPUHBCdDgtX0I3NDR0TzNFYXFiZWdaT0x2ekxVSC00eVBhT1J5ZC12ZlZXb0dkVGU0YTBrelFMNHJKWWRuZ2tVdDVqdkFHVFAzU3hNM0NoczBkV1NtNzgxVHZRLWNialIxUEx3a0ZEREdQSE56MXhYY3RVSlp5Q1AwT2Jiekpya3ZQYzd2eHAwVG9wYWpMSUM5WVROYWJGaWNEMHg2MXYxdmcyLUVQV011NGdzOElKZ1BLQkp0RjB3cjVhNUlLV2Zv?oc=5</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" s="1" t="n">
+        <v>46055.79517361111</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>(technology OR cybersecurity OR ransomware OR hacking OR AI OR "artificial intelligence" OR "machine learning" OR automation OR quantum OR semiconductor OR software OR cloud OR 5G OR robotics) AND (launch OR update OR vulnerability OR breach OR research OR earnings OR partnership OR regulation) -(rumor OR review OR gaming OR crypto OR podcast OR live OR blog)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Palantir beats fourth-quarter estimates on the strength of AI and defense demand - CNBC</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 21:06:32 GMT</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE52amFPRG1pR1dBclY2VlpPYU85dWNkaFFHRGw4REVNT0hqM2o0NVJhR1BHWHlLNFFpUVA1dVZJN2dpZEIzcGRuVE1pdkxqazRjZGtSNkMtWGdIZ1MxWXl4VGZueHBHTDRmMFQwR0JVdThvTTVmOVHSAXtBVV95cUxOWnpvU2RBSG1qVkdDLVY2MGpoU0thN0prd3VIc0puMllkX3VfdE51RW9GampfcVdmTnVaLTFHSlg3R0xFd081S0hxdy1uXzEtZlBPY0l2dnF5amMwWnlxQm9pM19YeHpzOTAxdVBfSzF1NHpKUGVMcXpfNTQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="1" t="n">
+        <v>46055.87953703704</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>Fraud_Scam</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Scam emails claiming to be from Okotoks Oilers still circulating - OkotoksOnline</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Mon, 02 Feb 2026 12:06:07 GMT</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNQ0txZE1iWXdHNlJjNVRKQ3g2SEN3YmJBdWNLTjd6RDJYbFMzYV9lYTJsZ1NUY1pCbmJ2REJ2YUxXQ1FtNXhCa3VCNDJfUmpGMGM4dnlaTTFvMnFXbF9VTlR0NzgxcWxYcGphclFISDFJZi1EVDUwd3BaWmY0NkY4V09wa0dzQ211TXpEV19uY1JSOWFxQlMxQjZ4SG41SjBY?oc=5</t>
-        </is>
-      </c>
-      <c r="F91" t="n">
-        <v>1</v>
-      </c>
-      <c r="G91" s="1" t="n">
-        <v>46055.50424768519</v>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Syncro Marketplace Now Offering IRONSCALES Email Security Services to MSPs - ChannelE2E</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 14:00:00 GMT</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNUVYzWi1sSDk4QUF6TGFDa2QwTXl4SlNoT0dnajh3SmF4OEJud0NTRF8ySkk1NmNRVE1DT3d2UEZJNGltTGpjWEUxT0xJTXBvTktjb2lPd1pRZnk2RVJfYWhnSkZxRF9vOGRVUHpmNVNTLXJodEx6WWo2cXFBdmdTcE81bnlJZGtqWmtSVUp1cGN6LTc5NHBjTmJnVXM4UnZnc21ieXNDcmZ6UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="1" t="n">
+        <v>46055.58333333334</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Fraud_Scam</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Scam Alert: Muscatine warns of planning and zoning impersonation - KWQC</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 20:48:00 GMT</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxNVlJDQlRHWi14dHpfMWhEaVVjdU1vSGpoa3V1S2FCRnprTUNQZE1fRVZlMmFvNEp3RVgzanQwc2hCOFpoNk5QaVBFMmNkOGJxMy00WkV6VGZOYjhCMG94MG5fSVJSdU5IWXhhODlWVjVhV1JYUFlPZmJWNm1wQlcxVTBOZl93WDhibXJqQUNDczZ1ejjSAacBQVVfeXFMTlhDV1ZnMzQwcExSeWswVURrTm9fVW9uSnRGdVpON0RZYjl4bUduaUFGN29NMUdCOTVKQlJDTzRMQ25OazVvYnI1OURmaTNQNElRMjZtX1NnSlUwZGVuWm9aSnluT0lqVW1ucUl4dGVkR0FQWjFYaEZKeUY5cS13bmZ0UVZpLU5YbWV6bjdWTXdvQXN2SEV6UXpJbVBiaUxpV3ZoaEY5dms?oc=5</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" s="1" t="n">
+        <v>46055.86666666667</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Fraud_Scam</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Phishing Scam Uses Clean Emails and PDFs to Steal Dropbox Logins - Hackread</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 19:31:17 GMT</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBmQ3hleDhQc3dBbEFOWUNxdC1MbG9Gb1RWaUwydUp6M1hXOTFyUENQbEpZVWVxNEtGcmVJRDlsVWI4QjFLT3lYNUtSbmtHVjFMdVdFcFBvbkxMcllWeEQtdHB0ZjYwclR3Smc4QU5MOWxWVTBOQnZv?oc=5</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" s="1" t="n">
+        <v>46055.8133912037</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Fraud_Scam</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>(fraud OR scam OR phishing OR smishing OR vishing OR "identity theft" OR impersonation OR spoofing OR "account takeover" OR "payment fraud" OR "invoice fraud" OR "wire fraud" OR "business email compromise" OR BEC OR "fake invoice" OR "supplier fraud" OR "procurement fraud" OR "social engineering" OR extortion OR blackmail)AND (company OR business OR enterprise OR customer OR client OR employee OR bank OR financial OR payment OR transaction)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Scam emails claiming to be from Okotoks Oilers still circulating - HighRiverOnline</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Mon, 02 Feb 2026 12:03:44 GMT</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOaXFHaERNMEctdnA5ZWloTUlKdWxheW1Yd0R1cWdLVVMxNlhjWFRVQm8xVXBzaVJqbHl6SlhGZTJONXctcDJPVXpuclNyR0R4dGpnZXJPSGR0TTd4ZlZsRjZHeFJzOURiUkNDNVFVNDVhZkwwVkZGcmhxLXpNSE43NzcwVTFwLXBxaEwybWNIZTR5ZW9qQVdsVEZqQWhPVjJteHNZ?oc=5</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" s="1" t="n">
+        <v>46055.50259259259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>